<commit_message>
UI Overhaul: Implemented Premium Glass UI v3.0, restored management reports, synced May sales data, and added Daily Log view
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F185"/>
+  <dimension ref="A1:F186"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1223,10 +1223,10 @@
         <v>Mar26</v>
       </c>
       <c r="C5" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D5" t="str">
-        <v>Fixed Costs</v>
+        <v>Water</v>
       </c>
       <c r="E5" t="str">
         <v>Unknown</v>
@@ -3643,10 +3643,10 @@
         <v>Apr26</v>
       </c>
       <c r="C126" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D126" t="str">
-        <v>Other</v>
+        <v>Water</v>
       </c>
       <c r="E126" t="str">
         <v>น้ำ500</v>
@@ -4077,7 +4077,7 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>16/04/2026</v>
+        <v>18/04/2026</v>
       </c>
       <c r="B148" t="str">
         <v>Apr26</v>
@@ -4086,13 +4086,13 @@
         <v>COGS</v>
       </c>
       <c r="D148" t="str">
-        <v>Ice</v>
+        <v>Apple/Melon</v>
       </c>
       <c r="E148" t="str">
-        <v>เครื่องสกัดเย็น 2 เครื่องร้านใหม่</v>
+        <v>แอปเปิ้ล 3 ลัง</v>
       </c>
       <c r="F148">
-        <v>11560</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="149">
@@ -4106,13 +4106,13 @@
         <v>COGS</v>
       </c>
       <c r="D149" t="str">
-        <v>Orange</v>
+        <v>Mango</v>
       </c>
       <c r="E149" t="str">
-        <v>ลงทุนน้ำส้ม</v>
+        <v>16/04/26 มะม่วง 1 ลัง</v>
       </c>
       <c r="F149">
-        <v>9341</v>
+        <v>750</v>
       </c>
     </row>
     <row r="150">
@@ -4123,21 +4123,21 @@
         <v>Apr26</v>
       </c>
       <c r="C150" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D150" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E150" t="str">
-        <v>ค่าปริ้นgrcode</v>
+        <v>16/4/2569</v>
       </c>
       <c r="F150">
-        <v>60</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>18/04/2026</v>
+        <v>20/04/2026</v>
       </c>
       <c r="B151" t="str">
         <v>Apr26</v>
@@ -4146,18 +4146,18 @@
         <v>COGS</v>
       </c>
       <c r="D151" t="str">
-        <v>Apple/Melon</v>
+        <v>Orange</v>
       </c>
       <c r="E151" t="str">
-        <v>แอปเปิ้ล 3 ลัง</v>
+        <v>ส้ม 40 ตะกร้า ตะกร้าละ 22 โล โลละ 30 บาท</v>
       </c>
       <c r="F151">
-        <v>1050</v>
+        <v>28600</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>18/04/2026</v>
+        <v>20/04/2026</v>
       </c>
       <c r="B152" t="str">
         <v>Apr26</v>
@@ -4166,33 +4166,33 @@
         <v>COGS</v>
       </c>
       <c r="D152" t="str">
-        <v>Mango</v>
+        <v>Transportation</v>
       </c>
       <c r="E152" t="str">
-        <v>16/04/26 มะม่วง 1 ลัง</v>
+        <v>ค่าส่งป้ายเมนูร้านใหม่</v>
       </c>
       <c r="F152">
-        <v>750</v>
+        <v>335</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>18/04/2026</v>
+        <v>20/04/2026</v>
       </c>
       <c r="B153" t="str">
         <v>Apr26</v>
       </c>
       <c r="C153" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D153" t="str">
-        <v>Other</v>
+        <v>Packaging</v>
       </c>
       <c r="E153" t="str">
-        <v>16/4/2569</v>
+        <v>ขวดใหญ่ 98 อัน</v>
       </c>
       <c r="F153">
-        <v>4000</v>
+        <v>338</v>
       </c>
     </row>
     <row r="154">
@@ -4206,13 +4206,13 @@
         <v>COGS</v>
       </c>
       <c r="D154" t="str">
-        <v>Orange</v>
+        <v>Packaging</v>
       </c>
       <c r="E154" t="str">
-        <v>ส้ม 40 ตะกร้า ตะกร้าละ 22 โล โลละ 30 บาท</v>
+        <v>ถุงขยะ 10 แพค</v>
       </c>
       <c r="F154">
-        <v>28600</v>
+        <v>520</v>
       </c>
     </row>
     <row r="155">
@@ -4226,13 +4226,13 @@
         <v>COGS</v>
       </c>
       <c r="D155" t="str">
-        <v>Transportation</v>
+        <v>Watermelon</v>
       </c>
       <c r="E155" t="str">
-        <v>ค่าส่งป้ายเมนูร้านใหม่</v>
+        <v>18/4/26 แตงโม 30 ลูก</v>
       </c>
       <c r="F155">
-        <v>335</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="156">
@@ -4246,18 +4246,18 @@
         <v>COGS</v>
       </c>
       <c r="D156" t="str">
-        <v>Packaging</v>
+        <v>Mango</v>
       </c>
       <c r="E156" t="str">
-        <v>ขวดใหญ่ 98 อัน</v>
+        <v>18/4/26 มะม่วง 25 โล 750</v>
       </c>
       <c r="F156">
-        <v>338</v>
+        <v>750</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>20/04/2026</v>
+        <v>21/04/2026</v>
       </c>
       <c r="B157" t="str">
         <v>Apr26</v>
@@ -4266,18 +4266,18 @@
         <v>COGS</v>
       </c>
       <c r="D157" t="str">
-        <v>Packaging</v>
+        <v>Watermelon</v>
       </c>
       <c r="E157" t="str">
-        <v>ถุงขยะ 10 แพค</v>
+        <v>21/4/26 แตงโม60 ลูก</v>
       </c>
       <c r="F157">
-        <v>520</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>20/04/2026</v>
+        <v>21/04/2026</v>
       </c>
       <c r="B158" t="str">
         <v>Apr26</v>
@@ -4286,18 +4286,18 @@
         <v>COGS</v>
       </c>
       <c r="D158" t="str">
-        <v>Watermelon</v>
+        <v>Transportation</v>
       </c>
       <c r="E158" t="str">
-        <v>18/4/26 แตงโม 30 ลูก</v>
+        <v>Lalamove</v>
       </c>
       <c r="F158">
-        <v>2400</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>20/04/2026</v>
+        <v>21/04/2026</v>
       </c>
       <c r="B159" t="str">
         <v>Apr26</v>
@@ -4306,18 +4306,18 @@
         <v>COGS</v>
       </c>
       <c r="D159" t="str">
-        <v>Mango</v>
+        <v>Apple/Melon</v>
       </c>
       <c r="E159" t="str">
-        <v>18/4/26 มะม่วง 25 โล 750</v>
+        <v>แอปเปิ้ล 4 ลัง</v>
       </c>
       <c r="F159">
-        <v>750</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>20/04/2026</v>
+        <v>23/04/2026</v>
       </c>
       <c r="B160" t="str">
         <v>Apr26</v>
@@ -4326,18 +4326,18 @@
         <v>COGS</v>
       </c>
       <c r="D160" t="str">
-        <v>Packaging</v>
+        <v>Mango</v>
       </c>
       <c r="E160" t="str">
-        <v>ฝาปิดกล่องใส่ผลไม้ 2 อัน</v>
+        <v>มะม่วง 2 ลัง</v>
       </c>
       <c r="F160">
-        <v>692</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>21/04/2026</v>
+        <v>23/04/2026</v>
       </c>
       <c r="B161" t="str">
         <v>Apr26</v>
@@ -4346,18 +4346,18 @@
         <v>COGS</v>
       </c>
       <c r="D161" t="str">
-        <v>Watermelon</v>
+        <v>Apple/Melon</v>
       </c>
       <c r="E161" t="str">
-        <v>21/4/26 แตงโม60 ลูก</v>
+        <v>แอปเปิ้ล 4 ลัง</v>
       </c>
       <c r="F161">
-        <v>4800</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>21/04/2026</v>
+        <v>23/04/2026</v>
       </c>
       <c r="B162" t="str">
         <v>Apr26</v>
@@ -4366,18 +4366,18 @@
         <v>COGS</v>
       </c>
       <c r="D162" t="str">
-        <v>Transportation</v>
+        <v>Ice</v>
       </c>
       <c r="E162" t="str">
-        <v>Lalamove</v>
+        <v>16/4/26 เนื้อ 10 น้ำ 10 21/4/26 เนื้อ 10</v>
       </c>
       <c r="F162">
-        <v>2000</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>21/04/2026</v>
+        <v>23/04/2026</v>
       </c>
       <c r="B163" t="str">
         <v>Apr26</v>
@@ -4386,18 +4386,18 @@
         <v>COGS</v>
       </c>
       <c r="D163" t="str">
-        <v>Apple/Melon</v>
+        <v>Mango</v>
       </c>
       <c r="E163" t="str">
-        <v>แอปเปิ้ล 4 ลัง</v>
+        <v>มะม่วง 1 ลัง</v>
       </c>
       <c r="F163">
-        <v>1400</v>
+        <v>780</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>23/04/2026</v>
+        <v>24/04/2026</v>
       </c>
       <c r="B164" t="str">
         <v>Apr26</v>
@@ -4406,18 +4406,18 @@
         <v>COGS</v>
       </c>
       <c r="D164" t="str">
-        <v>Mango</v>
+        <v>Packaging</v>
       </c>
       <c r="E164" t="str">
-        <v>มะม่วง 2 ลัง</v>
+        <v>บาร์เลย 4 ถั่วแดง 3 ถุงละ 60</v>
       </c>
       <c r="F164">
-        <v>1560</v>
+        <v>420</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>23/04/2026</v>
+        <v>24/04/2026</v>
       </c>
       <c r="B165" t="str">
         <v>Apr26</v>
@@ -4426,18 +4426,18 @@
         <v>COGS</v>
       </c>
       <c r="D165" t="str">
-        <v>Apple/Melon</v>
+        <v>Watermelon</v>
       </c>
       <c r="E165" t="str">
-        <v>แอปเปิ้ล 4 ลัง</v>
+        <v>แตงโม 50 ลูก</v>
       </c>
       <c r="F165">
-        <v>1400</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>23/04/2026</v>
+        <v>25/04/2026</v>
       </c>
       <c r="B166" t="str">
         <v>Apr26</v>
@@ -4446,18 +4446,18 @@
         <v>COGS</v>
       </c>
       <c r="D166" t="str">
-        <v>Ice</v>
+        <v>Orange</v>
       </c>
       <c r="E166" t="str">
-        <v>16/4/26 เนื้อ 10 น้ำ 10 21/4/26 เนื้อ 10</v>
+        <v>22/04/69</v>
       </c>
       <c r="F166">
-        <v>2900</v>
+        <v>14400</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>23/04/2026</v>
+        <v>26/04/2026</v>
       </c>
       <c r="B167" t="str">
         <v>Apr26</v>
@@ -4466,18 +4466,18 @@
         <v>COGS</v>
       </c>
       <c r="D167" t="str">
-        <v>Mango</v>
+        <v>Packaging</v>
       </c>
       <c r="E167" t="str">
-        <v>มะม่วง 1 ลัง</v>
+        <v>แก้ว 1 ลัง</v>
       </c>
       <c r="F167">
-        <v>780</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>24/04/2026</v>
+        <v>26/04/2026</v>
       </c>
       <c r="B168" t="str">
         <v>Apr26</v>
@@ -4489,15 +4489,15 @@
         <v>Packaging</v>
       </c>
       <c r="E168" t="str">
-        <v>บาร์เลย 4 ถั่วแดง 3 ถุงละ 60</v>
+        <v>แก้ว3ลัง</v>
       </c>
       <c r="F168">
-        <v>420</v>
+        <v>7090</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>24/04/2026</v>
+        <v>26/04/2026</v>
       </c>
       <c r="B169" t="str">
         <v>Apr26</v>
@@ -4506,18 +4506,18 @@
         <v>COGS</v>
       </c>
       <c r="D169" t="str">
-        <v>Watermelon</v>
+        <v>Mango</v>
       </c>
       <c r="E169" t="str">
-        <v>แตงโม 50 ลูก</v>
+        <v>มะม่วง 1 ลัง</v>
       </c>
       <c r="F169">
-        <v>4000</v>
+        <v>780</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>25/04/2026</v>
+        <v>26/04/2026</v>
       </c>
       <c r="B170" t="str">
         <v>Apr26</v>
@@ -4526,18 +4526,18 @@
         <v>COGS</v>
       </c>
       <c r="D170" t="str">
-        <v>Orange</v>
+        <v>Apple/Melon</v>
       </c>
       <c r="E170" t="str">
-        <v>22/04/69</v>
+        <v>แอปเปิ้ล 4</v>
       </c>
       <c r="F170">
-        <v>14400</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>25/04/2026</v>
+        <v>27/04/2026</v>
       </c>
       <c r="B171" t="str">
         <v>Apr26</v>
@@ -4549,15 +4549,15 @@
         <v>Ice</v>
       </c>
       <c r="E171" t="str">
-        <v>พัดลม 2 ตัว</v>
+        <v>26/4/26 50 ลูก</v>
       </c>
       <c r="F171">
-        <v>1838</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>26/04/2026</v>
+        <v>28/04/2026</v>
       </c>
       <c r="B172" t="str">
         <v>Apr26</v>
@@ -4569,15 +4569,15 @@
         <v>Packaging</v>
       </c>
       <c r="E172" t="str">
-        <v>แก้ว 1 ลัง</v>
+        <v>หลอด 704(20ห่อ)</v>
       </c>
       <c r="F172">
-        <v>1539</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>26/04/2026</v>
+        <v>28/04/2026</v>
       </c>
       <c r="B173" t="str">
         <v>Apr26</v>
@@ -4586,18 +4586,18 @@
         <v>COGS</v>
       </c>
       <c r="D173" t="str">
-        <v>Packaging</v>
+        <v>Orange</v>
       </c>
       <c r="E173" t="str">
-        <v>แก้ว3ลัง</v>
+        <v>รอบ 27/04/69</v>
       </c>
       <c r="F173">
-        <v>7090</v>
+        <v>21600</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>26/04/2026</v>
+        <v>28/04/2026</v>
       </c>
       <c r="B174" t="str">
         <v>Apr26</v>
@@ -4606,18 +4606,18 @@
         <v>COGS</v>
       </c>
       <c r="D174" t="str">
-        <v>Mango</v>
+        <v>Coconut</v>
       </c>
       <c r="E174" t="str">
-        <v>มะม่วง 1 ลัง</v>
+        <v>ค่าส่งมะพร้าว</v>
       </c>
       <c r="F174">
-        <v>780</v>
+        <v>100</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>26/04/2026</v>
+        <v>28/04/2026</v>
       </c>
       <c r="B175" t="str">
         <v>Apr26</v>
@@ -4629,7 +4629,7 @@
         <v>Apple/Melon</v>
       </c>
       <c r="E175" t="str">
-        <v>แอปเปิ้ล 4</v>
+        <v>แอปเปิ้ล 4 ลัง</v>
       </c>
       <c r="F175">
         <v>1400</v>
@@ -4637,7 +4637,7 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>27/04/2026</v>
+        <v>28/04/2026</v>
       </c>
       <c r="B176" t="str">
         <v>Apr26</v>
@@ -4646,18 +4646,18 @@
         <v>COGS</v>
       </c>
       <c r="D176" t="str">
-        <v>Ice</v>
+        <v>Mango</v>
       </c>
       <c r="E176" t="str">
-        <v>26/4/26 50 ลูก</v>
+        <v>มะม่วง 2 ลัง</v>
       </c>
       <c r="F176">
-        <v>4000</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>28/04/2026</v>
+        <v>29/04/2026</v>
       </c>
       <c r="B177" t="str">
         <v>Apr26</v>
@@ -4666,18 +4666,18 @@
         <v>COGS</v>
       </c>
       <c r="D177" t="str">
-        <v>Packaging</v>
+        <v>Milk/Conden</v>
       </c>
       <c r="E177" t="str">
-        <v>หลอด 704(20ห่อ)</v>
+        <v>นมข้นหวาน1ลัง 836</v>
       </c>
       <c r="F177">
-        <v>2110</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>28/04/2026</v>
+        <v>29/04/2026</v>
       </c>
       <c r="B178" t="str">
         <v>Apr26</v>
@@ -4686,18 +4686,18 @@
         <v>COGS</v>
       </c>
       <c r="D178" t="str">
-        <v>Orange</v>
+        <v>Packaging</v>
       </c>
       <c r="E178" t="str">
-        <v>รอบ 27/04/69</v>
+        <v>นมข้นหวาน2ลัง 1602</v>
       </c>
       <c r="F178">
-        <v>21600</v>
+        <v>3210</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>28/04/2026</v>
+        <v>29/04/2026</v>
       </c>
       <c r="B179" t="str">
         <v>Apr26</v>
@@ -4706,18 +4706,18 @@
         <v>COGS</v>
       </c>
       <c r="D179" t="str">
-        <v>Coconut</v>
+        <v>Watermelon</v>
       </c>
       <c r="E179" t="str">
-        <v>ค่าส่งมะพร้าว</v>
+        <v>แตงโม 60 ลูก</v>
       </c>
       <c r="F179">
-        <v>100</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>28/04/2026</v>
+        <v>29/04/2026</v>
       </c>
       <c r="B180" t="str">
         <v>Apr26</v>
@@ -4726,18 +4726,18 @@
         <v>COGS</v>
       </c>
       <c r="D180" t="str">
-        <v>Apple/Melon</v>
+        <v>Transportation</v>
       </c>
       <c r="E180" t="str">
-        <v>แอปเปิ้ล 4 ลัง</v>
+        <v>เนื้อ 10 x 50 500</v>
       </c>
       <c r="F180">
-        <v>1400</v>
+        <v>2395</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>28/04/2026</v>
+        <v>30/04/2026</v>
       </c>
       <c r="B181" t="str">
         <v>Apr26</v>
@@ -4746,18 +4746,18 @@
         <v>COGS</v>
       </c>
       <c r="D181" t="str">
-        <v>Mango</v>
+        <v>Ice</v>
       </c>
       <c r="E181" t="str">
-        <v>มะม่วง 2 ลัง</v>
+        <v>สับปะรส 3 ตะกร้า</v>
       </c>
       <c r="F181">
-        <v>1560</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>29/04/2026</v>
+        <v>30/04/2026</v>
       </c>
       <c r="B182" t="str">
         <v>Apr26</v>
@@ -4766,78 +4766,98 @@
         <v>OPEX</v>
       </c>
       <c r="D182" t="str">
-        <v>Other</v>
+        <v>Salary</v>
       </c>
       <c r="E182" t="str">
-        <v>นมข้นหวาน1ลัง 836</v>
+        <v>Employee 1</v>
       </c>
       <c r="F182">
-        <v>2160</v>
+        <v>19000</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>29/04/2026</v>
+        <v>30/04/2026</v>
       </c>
       <c r="B183" t="str">
         <v>Apr26</v>
       </c>
       <c r="C183" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D183" t="str">
-        <v>Packaging</v>
+        <v>Salary</v>
       </c>
       <c r="E183" t="str">
-        <v>นมข้นหวาน2ลัง 1602</v>
+        <v>Employee 2</v>
       </c>
       <c r="F183">
-        <v>3210</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>29/04/2026</v>
+        <v>30/04/2026</v>
       </c>
       <c r="B184" t="str">
         <v>Apr26</v>
       </c>
       <c r="C184" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D184" t="str">
-        <v>Watermelon</v>
+        <v>Fixed Costs</v>
       </c>
       <c r="E184" t="str">
-        <v>แตงโม 60 ลูก</v>
+        <v>Rent</v>
       </c>
       <c r="F184">
-        <v>4200</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>29/04/2026</v>
+        <v>30/04/2026</v>
       </c>
       <c r="B185" t="str">
         <v>Apr26</v>
       </c>
       <c r="C185" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D185" t="str">
-        <v>Transportation</v>
+        <v>Investment</v>
       </c>
       <c r="E185" t="str">
-        <v>เนื้อ 10 x 50 500</v>
+        <v>Stock (Allocated 82.9%)</v>
       </c>
       <c r="F185">
-        <v>2395</v>
+        <v>9948</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>30/04/2026</v>
+      </c>
+      <c r="B186" t="str">
+        <v>Apr26</v>
+      </c>
+      <c r="C186" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D186" t="str">
+        <v>Other</v>
+      </c>
+      <c r="E186" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="F186">
+        <v>1500</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F185"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F186"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11091,7 +11111,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z34"/>
+  <dimension ref="A1:Z35"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11192,22 +11212,22 @@
         <v>6300</v>
       </c>
       <c r="E3">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>6180</v>
+        <v>6300</v>
       </c>
       <c r="G3">
-        <v>4180</v>
+        <v>4280</v>
       </c>
       <c r="H3">
         <v>92</v>
       </c>
       <c r="I3">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="K3">
         <v>6</v>
@@ -11225,7 +11245,7 @@
         <v>0</v>
       </c>
       <c r="P3">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -11352,10 +11372,10 @@
         <v>9930</v>
       </c>
       <c r="E5">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>9750</v>
+        <v>9930</v>
       </c>
       <c r="G5">
         <v>4690</v>
@@ -11364,7 +11384,7 @@
         <v>81</v>
       </c>
       <c r="I5">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>48</v>
@@ -11379,7 +11399,7 @@
         <v>15</v>
       </c>
       <c r="N5">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -11394,7 +11414,7 @@
         <v>0</v>
       </c>
       <c r="S5">
-        <v>7.5</v>
+        <v>2.5</v>
       </c>
       <c r="T5">
         <v>11</v>
@@ -11403,16 +11423,16 @@
         <v>0</v>
       </c>
       <c r="V5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z5">
         <v>0</v>
@@ -11512,10 +11532,10 @@
         <v>9540</v>
       </c>
       <c r="E7">
-        <v>240</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>9300</v>
+        <v>9540</v>
       </c>
       <c r="G7">
         <v>7560</v>
@@ -11524,7 +11544,7 @@
         <v>100</v>
       </c>
       <c r="I7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>68</v>
@@ -11533,13 +11553,13 @@
         <v>17</v>
       </c>
       <c r="L7">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="M7">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="N7">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O7">
         <v>0</v>
@@ -11563,16 +11583,16 @@
         <v>34</v>
       </c>
       <c r="V7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z7">
         <v>28</v>
@@ -11592,10 +11612,10 @@
         <v>8510</v>
       </c>
       <c r="E8">
-        <v>240</v>
+        <v>0</v>
       </c>
       <c r="F8">
-        <v>8270</v>
+        <v>8510</v>
       </c>
       <c r="G8">
         <v>4100</v>
@@ -11604,7 +11624,7 @@
         <v>64</v>
       </c>
       <c r="I8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <v>70</v>
@@ -11619,7 +11639,7 @@
         <v>8</v>
       </c>
       <c r="N8">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="O8">
         <v>0</v>
@@ -11643,16 +11663,16 @@
         <v>32</v>
       </c>
       <c r="V8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z8">
         <v>16</v>
@@ -11672,10 +11692,10 @@
         <v>6420</v>
       </c>
       <c r="E9">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>6240</v>
+        <v>6420</v>
       </c>
       <c r="G9">
         <v>3180</v>
@@ -11684,7 +11704,7 @@
         <v>56</v>
       </c>
       <c r="I9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J9">
         <v>32</v>
@@ -11699,7 +11719,7 @@
         <v>9</v>
       </c>
       <c r="N9">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="O9">
         <v>0</v>
@@ -11720,22 +11740,22 @@
         <v>11</v>
       </c>
       <c r="U9">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="V9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z9">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -11752,10 +11772,10 @@
         <v>6180</v>
       </c>
       <c r="E10">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F10">
-        <v>6000</v>
+        <v>6180</v>
       </c>
       <c r="G10">
         <v>2880</v>
@@ -11764,7 +11784,7 @@
         <v>49</v>
       </c>
       <c r="I10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J10">
         <v>55</v>
@@ -11779,7 +11799,7 @@
         <v>6</v>
       </c>
       <c r="N10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O10">
         <v>0</v>
@@ -11800,22 +11820,22 @@
         <v>17</v>
       </c>
       <c r="U10">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="V10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z10">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -11832,10 +11852,10 @@
         <v>5090</v>
       </c>
       <c r="E11">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>4970</v>
+        <v>5090</v>
       </c>
       <c r="G11">
         <v>3130</v>
@@ -11844,7 +11864,7 @@
         <v>64</v>
       </c>
       <c r="I11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J11">
         <v>37</v>
@@ -11859,7 +11879,7 @@
         <v>7</v>
       </c>
       <c r="N11">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O11">
         <v>0</v>
@@ -11880,7 +11900,7 @@
         <v>9</v>
       </c>
       <c r="U11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V11">
         <v>0</v>
@@ -11895,7 +11915,7 @@
         <v>0</v>
       </c>
       <c r="Z11">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -11912,10 +11932,10 @@
         <v>9150</v>
       </c>
       <c r="E12">
-        <v>240</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>8910</v>
+        <v>9150</v>
       </c>
       <c r="G12">
         <v>4890</v>
@@ -11924,7 +11944,7 @@
         <v>58</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J12">
         <v>63</v>
@@ -11939,7 +11959,7 @@
         <v>22</v>
       </c>
       <c r="N12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O12">
         <v>0</v>
@@ -11963,16 +11983,16 @@
         <v>0</v>
       </c>
       <c r="V12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z12">
         <v>0</v>
@@ -11992,10 +12012,10 @@
         <v>10880</v>
       </c>
       <c r="E13">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>10700</v>
+        <v>10880</v>
       </c>
       <c r="G13">
         <v>5620</v>
@@ -12004,7 +12024,7 @@
         <v>60</v>
       </c>
       <c r="I13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J13">
         <v>85</v>
@@ -12040,22 +12060,22 @@
         <v>21</v>
       </c>
       <c r="U13">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="V13">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W13">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z13">
-        <v>0</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
@@ -12072,10 +12092,10 @@
         <v>9460</v>
       </c>
       <c r="E14">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>9280</v>
+        <v>9460</v>
       </c>
       <c r="G14">
         <v>4680</v>
@@ -12084,7 +12104,7 @@
         <v>82</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J14">
         <v>79</v>
@@ -12123,16 +12143,16 @@
         <v>18</v>
       </c>
       <c r="V14">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W14">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X14">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y14">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z14">
         <v>26</v>
@@ -12152,10 +12172,10 @@
         <v>7180</v>
       </c>
       <c r="E15">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F15">
-        <v>7000</v>
+        <v>7180</v>
       </c>
       <c r="G15">
         <v>3630</v>
@@ -12164,7 +12184,7 @@
         <v>65</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J15">
         <v>67</v>
@@ -12203,16 +12223,16 @@
         <v>0</v>
       </c>
       <c r="V15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z15">
         <v>0</v>
@@ -12232,10 +12252,10 @@
         <v>10980</v>
       </c>
       <c r="E16">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>10800</v>
+        <v>10980</v>
       </c>
       <c r="G16">
         <v>4200</v>
@@ -12244,7 +12264,7 @@
         <v>100</v>
       </c>
       <c r="I16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J16">
         <v>62</v>
@@ -12283,16 +12303,16 @@
         <v>12</v>
       </c>
       <c r="V16">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W16">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z16">
         <v>0</v>
@@ -12472,10 +12492,10 @@
         <v>6560</v>
       </c>
       <c r="E19">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F19">
-        <v>6380</v>
+        <v>6560</v>
       </c>
       <c r="G19">
         <v>3990</v>
@@ -12484,7 +12504,7 @@
         <v>78</v>
       </c>
       <c r="I19">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J19">
         <v>40</v>
@@ -12523,16 +12543,16 @@
         <v>14</v>
       </c>
       <c r="V19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z19">
         <v>0</v>
@@ -12552,10 +12572,10 @@
         <v>5920</v>
       </c>
       <c r="E20">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F20">
-        <v>5800</v>
+        <v>5920</v>
       </c>
       <c r="G20">
         <v>5120</v>
@@ -12603,16 +12623,16 @@
         <v>10</v>
       </c>
       <c r="V20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z20">
         <v>22</v>
@@ -12632,10 +12652,10 @@
         <v>3870</v>
       </c>
       <c r="E21">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F21">
-        <v>3750</v>
+        <v>3870</v>
       </c>
       <c r="G21">
         <v>2630</v>
@@ -12683,16 +12703,16 @@
         <v>0</v>
       </c>
       <c r="V21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z21">
         <v>8</v>
@@ -12712,10 +12732,10 @@
         <v>4670</v>
       </c>
       <c r="E22">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F22">
-        <v>4520</v>
+        <v>4670</v>
       </c>
       <c r="G22">
         <v>5220</v>
@@ -12763,16 +12783,16 @@
         <v>18</v>
       </c>
       <c r="V22">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W22">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="X22">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y22">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z22">
         <v>16</v>
@@ -12792,10 +12812,10 @@
         <v>5470</v>
       </c>
       <c r="E23">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F23">
-        <v>5350</v>
+        <v>5470</v>
       </c>
       <c r="G23">
         <v>3200</v>
@@ -12843,16 +12863,16 @@
         <v>10</v>
       </c>
       <c r="V23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Z23">
         <v>34</v>
@@ -13352,10 +13372,10 @@
         <v>4980</v>
       </c>
       <c r="E30">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F30">
-        <v>4860</v>
+        <v>4980</v>
       </c>
       <c r="G30">
         <v>3040</v>
@@ -13384,14 +13404,23 @@
       <c r="O30">
         <v>0</v>
       </c>
+      <c r="P30">
+        <v>130</v>
+      </c>
       <c r="Q30">
         <v>0</v>
       </c>
       <c r="R30">
         <v>0</v>
       </c>
+      <c r="S30">
+        <v>1</v>
+      </c>
+      <c r="T30">
+        <v>18</v>
+      </c>
       <c r="U30">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V30">
         <v>0</v>
@@ -13406,7 +13435,7 @@
         <v>0</v>
       </c>
       <c r="Z30">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31">
@@ -13480,238 +13509,1357 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="B33" t="str">
-        <v>29 days</v>
-      </c>
-      <c r="C33">
-        <v>303628</v>
-      </c>
-      <c r="D33">
-        <v>186770</v>
-      </c>
-      <c r="E33">
-        <v>4680</v>
-      </c>
-      <c r="F33">
-        <v>182090</v>
-      </c>
-      <c r="G33">
-        <v>116858</v>
-      </c>
-      <c r="H33">
-        <v>1845</v>
-      </c>
-      <c r="I33">
-        <v>67</v>
-      </c>
-      <c r="J33">
-        <v>1400</v>
-      </c>
-      <c r="K33">
-        <v>221</v>
-      </c>
-      <c r="L33">
-        <v>1325</v>
-      </c>
-      <c r="M33">
-        <v>258</v>
-      </c>
-      <c r="N33">
-        <v>57</v>
-      </c>
-      <c r="O33">
-        <v>0</v>
-      </c>
-      <c r="P33">
-        <v>4798</v>
-      </c>
-      <c r="Q33">
-        <v>0</v>
-      </c>
-      <c r="R33">
-        <v>0</v>
-      </c>
-      <c r="S33">
-        <v>72</v>
-      </c>
-      <c r="T33">
-        <v>349</v>
-      </c>
-      <c r="U33">
-        <v>282</v>
-      </c>
-      <c r="V33">
-        <v>52</v>
-      </c>
-      <c r="W33">
-        <v>54</v>
-      </c>
-      <c r="X33">
-        <v>32.5</v>
-      </c>
-      <c r="Y33">
-        <v>45</v>
-      </c>
-      <c r="Z33">
-        <v>316</v>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>30/04/2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C32">
+        <v>10230</v>
+      </c>
+      <c r="D32">
+        <v>6250</v>
+      </c>
+      <c r="E32">
+        <v>210</v>
+      </c>
+      <c r="F32">
+        <v>6040</v>
+      </c>
+      <c r="G32">
+        <v>3980</v>
+      </c>
+      <c r="H32">
+        <v>48</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>60</v>
+      </c>
+      <c r="K32">
+        <v>5</v>
+      </c>
+      <c r="L32">
+        <v>51</v>
+      </c>
+      <c r="M32">
+        <v>14</v>
+      </c>
+      <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
+        <v>0</v>
+      </c>
+      <c r="P32">
+        <v>178</v>
+      </c>
+      <c r="Q32">
+        <v>0</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+      <c r="U32">
+        <v>0</v>
+      </c>
+      <c r="V32">
+        <v>0</v>
+      </c>
+      <c r="W32">
+        <v>0</v>
+      </c>
+      <c r="X32">
+        <v>0</v>
+      </c>
+      <c r="Y32">
+        <v>0</v>
+      </c>
+      <c r="Z32">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B34" t="str">
+        <v>30 days</v>
+      </c>
+      <c r="C34">
+        <v>313858</v>
+      </c>
+      <c r="D34">
+        <v>193020</v>
+      </c>
+      <c r="E34">
+        <v>1860</v>
+      </c>
+      <c r="F34">
+        <v>191160</v>
+      </c>
+      <c r="G34">
+        <v>120938</v>
+      </c>
+      <c r="H34">
+        <v>1893</v>
+      </c>
+      <c r="I34">
+        <v>15</v>
+      </c>
+      <c r="J34">
+        <v>1454</v>
+      </c>
+      <c r="K34">
+        <v>226</v>
+      </c>
+      <c r="L34">
+        <v>1366</v>
+      </c>
+      <c r="M34">
+        <v>282</v>
+      </c>
+      <c r="N34">
+        <v>9</v>
+      </c>
+      <c r="O34">
+        <v>0</v>
+      </c>
+      <c r="P34">
+        <v>5100</v>
+      </c>
+      <c r="Q34">
+        <v>0</v>
+      </c>
+      <c r="R34">
+        <v>0</v>
+      </c>
+      <c r="S34">
+        <v>68</v>
+      </c>
+      <c r="T34">
+        <v>367</v>
+      </c>
+      <c r="U34">
+        <v>372</v>
+      </c>
+      <c r="V34">
+        <v>19</v>
+      </c>
+      <c r="W34">
+        <v>19</v>
+      </c>
+      <c r="X34">
+        <v>11.5</v>
+      </c>
+      <c r="Y34">
+        <v>19</v>
+      </c>
+      <c r="Z34">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
         <v>AVG/DAY</v>
       </c>
-      <c r="C34">
-        <v>10469.931034482759</v>
-      </c>
-      <c r="D34">
-        <v>6440.3448275862065</v>
-      </c>
-      <c r="E34">
-        <v>161.3793103448276</v>
-      </c>
-      <c r="F34">
-        <v>6278.9655172413795</v>
-      </c>
-      <c r="G34">
-        <v>4029.5862068965516</v>
-      </c>
-      <c r="H34">
-        <v>63.62068965517241</v>
-      </c>
-      <c r="I34">
-        <v>2.310344827586207</v>
-      </c>
-      <c r="J34">
-        <v>48.275862068965516</v>
-      </c>
-      <c r="K34">
-        <v>7.620689655172414</v>
-      </c>
-      <c r="L34">
-        <v>45.689655172413794</v>
-      </c>
-      <c r="M34">
-        <v>8.89655172413793</v>
-      </c>
-      <c r="N34">
-        <v>1.9655172413793103</v>
-      </c>
-      <c r="O34">
-        <v>0</v>
-      </c>
-      <c r="P34">
-        <v>165.44827586206895</v>
-      </c>
-      <c r="Q34">
-        <v>0</v>
-      </c>
-      <c r="R34">
-        <v>0</v>
-      </c>
-      <c r="S34">
-        <v>2.4827586206896552</v>
-      </c>
-      <c r="T34">
-        <v>12.03448275862069</v>
-      </c>
-      <c r="U34">
-        <v>9.724137931034482</v>
-      </c>
-      <c r="V34">
-        <v>1.793103448275862</v>
-      </c>
-      <c r="W34">
-        <v>1.8620689655172413</v>
-      </c>
-      <c r="X34">
-        <v>1.1206896551724137</v>
-      </c>
-      <c r="Y34">
-        <v>1.5517241379310345</v>
-      </c>
-      <c r="Z34">
-        <v>10.89655172413793</v>
+      <c r="C35">
+        <v>10461.933333333332</v>
+      </c>
+      <c r="D35">
+        <v>6434</v>
+      </c>
+      <c r="E35">
+        <v>62</v>
+      </c>
+      <c r="F35">
+        <v>6372</v>
+      </c>
+      <c r="G35">
+        <v>4031.266666666667</v>
+      </c>
+      <c r="H35">
+        <v>63.1</v>
+      </c>
+      <c r="I35">
+        <v>0.5</v>
+      </c>
+      <c r="J35">
+        <v>48.46666666666667</v>
+      </c>
+      <c r="K35">
+        <v>7.533333333333333</v>
+      </c>
+      <c r="L35">
+        <v>45.53333333333333</v>
+      </c>
+      <c r="M35">
+        <v>9.4</v>
+      </c>
+      <c r="N35">
+        <v>0.3</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35">
+        <v>170</v>
+      </c>
+      <c r="Q35">
+        <v>0</v>
+      </c>
+      <c r="R35">
+        <v>0</v>
+      </c>
+      <c r="S35">
+        <v>2.2666666666666666</v>
+      </c>
+      <c r="T35">
+        <v>12.233333333333333</v>
+      </c>
+      <c r="U35">
+        <v>12.4</v>
+      </c>
+      <c r="V35">
+        <v>0.6333333333333333</v>
+      </c>
+      <c r="W35">
+        <v>0.6333333333333333</v>
+      </c>
+      <c r="X35">
+        <v>0.38333333333333336</v>
+      </c>
+      <c r="Y35">
+        <v>0.6333333333333333</v>
+      </c>
+      <c r="Z35">
+        <v>13.666666666666666</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z35"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:AD14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Som Sai Jai Cold Press Bar - May 2026</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Revenue (฿)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Cash (฿)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Expenses (฿)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Cash-Exp (฿)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Scan/Transfer (฿)</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Orange</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Orange (100)</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Watermelon</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Mango</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Coconut</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Apple</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Young Coco</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Total Cups</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Bot Big</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Bot Small</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Used Orange (basket)</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Used Watermelon (pcs)</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Used Mango</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Used Coco (Meat)</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Used Coco (Water)</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Used Coco (Conden)</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>Used Coco (Raw)</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>Used Apple</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>Used Guava</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>Used Pineapple</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>Used Young Coco</v>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Date</v>
+        <v>01/05/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>Day</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Revenue (฿)</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Cash (฿)</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Expenses (฿)</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Cash-Exp (฿)</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Scan/Transfer (฿)</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Orange</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Watermelon</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Mango</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Coconut</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Apple</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Young Coco</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Total Cups</v>
-      </c>
-      <c r="O3" t="str">
-        <v>Bot Big</v>
-      </c>
-      <c r="P3" t="str">
-        <v>Bot Small</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>Used Orange (basket)</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Used Watermelon (pcs)</v>
+        <v>Fri</v>
+      </c>
+      <c r="C3">
+        <v>13950</v>
+      </c>
+      <c r="D3">
+        <v>8220</v>
+      </c>
+      <c r="E3">
+        <v>180</v>
+      </c>
+      <c r="F3">
+        <v>8040</v>
+      </c>
+      <c r="G3">
+        <v>5730</v>
+      </c>
+      <c r="H3">
+        <v>81</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>57</v>
+      </c>
+      <c r="K3">
+        <v>8</v>
+      </c>
+      <c r="L3">
+        <v>72</v>
+      </c>
+      <c r="M3">
+        <v>15</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>233</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>3.5</v>
+      </c>
+      <c r="U3">
+        <v>15</v>
+      </c>
+      <c r="V3">
+        <v>16</v>
+      </c>
+      <c r="W3">
+        <v>4</v>
+      </c>
+      <c r="X3">
+        <v>4</v>
+      </c>
+      <c r="Y3">
+        <v>2</v>
+      </c>
+      <c r="Z3">
+        <v>4</v>
+      </c>
+      <c r="AA3">
+        <v>30</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>02/05/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C4">
+        <v>17070</v>
+      </c>
+      <c r="D4">
+        <v>9780</v>
+      </c>
+      <c r="E4">
+        <v>240</v>
+      </c>
+      <c r="F4">
+        <v>9540</v>
+      </c>
+      <c r="G4">
+        <v>7290</v>
+      </c>
+      <c r="H4">
+        <v>84</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>126</v>
+      </c>
+      <c r="K4">
+        <v>7</v>
+      </c>
+      <c r="L4">
+        <v>70</v>
+      </c>
+      <c r="M4">
+        <v>15</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>302</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>3.5</v>
+      </c>
+      <c r="U4">
+        <v>33</v>
+      </c>
+      <c r="V4">
+        <v>14</v>
+      </c>
+      <c r="W4">
+        <v>4</v>
+      </c>
+      <c r="X4">
+        <v>4</v>
+      </c>
+      <c r="Y4">
+        <v>2</v>
+      </c>
+      <c r="Z4">
+        <v>5</v>
+      </c>
+      <c r="AA4">
+        <v>30</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>03/05/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C5">
+        <v>12530</v>
+      </c>
+      <c r="D5">
+        <v>7520</v>
+      </c>
+      <c r="E5">
+        <v>180</v>
+      </c>
+      <c r="F5">
+        <v>7340</v>
+      </c>
+      <c r="G5">
+        <v>5010</v>
+      </c>
+      <c r="H5">
+        <v>63</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>70</v>
+      </c>
+      <c r="K5">
+        <v>5</v>
+      </c>
+      <c r="L5">
+        <v>67</v>
+      </c>
+      <c r="M5">
+        <v>13</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>218</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>2</v>
+      </c>
+      <c r="U5">
+        <v>18</v>
+      </c>
+      <c r="V5">
+        <v>10</v>
+      </c>
+      <c r="W5">
+        <v>4</v>
+      </c>
+      <c r="X5">
+        <v>4</v>
+      </c>
+      <c r="Y5">
+        <v>2</v>
+      </c>
+      <c r="Z5">
+        <v>4</v>
+      </c>
+      <c r="AA5">
+        <v>26</v>
+      </c>
+      <c r="AB5">
+        <v>0</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>04/05/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C6">
+        <v>10030</v>
+      </c>
+      <c r="D6">
+        <v>6400</v>
+      </c>
+      <c r="E6">
+        <v>180</v>
+      </c>
+      <c r="F6">
+        <v>6220</v>
+      </c>
+      <c r="G6">
+        <v>3630</v>
+      </c>
+      <c r="H6">
+        <v>43</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>68</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
+        <v>40</v>
+      </c>
+      <c r="M6">
+        <v>20</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>176</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>2</v>
+      </c>
+      <c r="U6">
+        <v>17</v>
+      </c>
+      <c r="V6">
+        <v>10</v>
+      </c>
+      <c r="W6">
+        <v>2</v>
+      </c>
+      <c r="X6">
+        <v>2</v>
+      </c>
+      <c r="Y6">
+        <v>1</v>
+      </c>
+      <c r="Z6">
+        <v>2</v>
+      </c>
+      <c r="AA6">
+        <v>40</v>
+      </c>
+      <c r="AB6">
+        <v>0</v>
+      </c>
+      <c r="AC6">
+        <v>0</v>
+      </c>
+      <c r="AD6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>05/05/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C7">
+        <v>7920</v>
+      </c>
+      <c r="D7">
+        <v>4400</v>
+      </c>
+      <c r="E7">
+        <v>120</v>
+      </c>
+      <c r="F7">
+        <v>4280</v>
+      </c>
+      <c r="G7">
+        <v>3520</v>
+      </c>
+      <c r="H7">
+        <v>28</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>60</v>
+      </c>
+      <c r="K7">
+        <v>4</v>
+      </c>
+      <c r="L7">
+        <v>39</v>
+      </c>
+      <c r="M7">
+        <v>9</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>140</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>1.5</v>
+      </c>
+      <c r="U7">
+        <v>15</v>
+      </c>
+      <c r="V7">
+        <v>8</v>
+      </c>
+      <c r="W7">
+        <v>2</v>
+      </c>
+      <c r="X7">
+        <v>2</v>
+      </c>
+      <c r="Y7">
+        <v>1</v>
+      </c>
+      <c r="Z7">
+        <v>2</v>
+      </c>
+      <c r="AA7">
+        <v>18</v>
+      </c>
+      <c r="AB7">
+        <v>0</v>
+      </c>
+      <c r="AC7">
+        <v>0</v>
+      </c>
+      <c r="AD7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>06/05/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C8">
+        <v>8830</v>
+      </c>
+      <c r="D8">
+        <v>4770</v>
+      </c>
+      <c r="E8">
+        <v>120</v>
+      </c>
+      <c r="F8">
+        <v>4650</v>
+      </c>
+      <c r="G8">
+        <v>4060</v>
+      </c>
+      <c r="H8">
+        <v>47</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>53</v>
+      </c>
+      <c r="K8">
+        <v>6</v>
+      </c>
+      <c r="L8">
+        <v>38</v>
+      </c>
+      <c r="M8">
+        <v>9</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>153</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>2.5</v>
+      </c>
+      <c r="U8">
+        <v>15</v>
+      </c>
+      <c r="V8">
+        <v>12</v>
+      </c>
+      <c r="W8">
+        <v>2</v>
+      </c>
+      <c r="X8">
+        <v>2</v>
+      </c>
+      <c r="Y8">
+        <v>1</v>
+      </c>
+      <c r="Z8">
+        <v>2</v>
+      </c>
+      <c r="AA8">
+        <v>18</v>
+      </c>
+      <c r="AB8">
+        <v>0</v>
+      </c>
+      <c r="AC8">
+        <v>0</v>
+      </c>
+      <c r="AD8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>07/05/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C9">
+        <v>5410</v>
+      </c>
+      <c r="D9">
+        <v>3010</v>
+      </c>
+      <c r="E9">
+        <v>120</v>
+      </c>
+      <c r="F9">
+        <v>2890</v>
+      </c>
+      <c r="G9">
+        <v>2400</v>
+      </c>
+      <c r="H9">
+        <v>37</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>26</v>
+      </c>
+      <c r="K9">
+        <v>3</v>
+      </c>
+      <c r="L9">
+        <v>20</v>
+      </c>
+      <c r="M9">
+        <v>7</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>93</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>2</v>
+      </c>
+      <c r="U9">
+        <v>8</v>
+      </c>
+      <c r="V9">
+        <v>6</v>
+      </c>
+      <c r="W9">
+        <v>1</v>
+      </c>
+      <c r="X9">
+        <v>1</v>
+      </c>
+      <c r="Y9">
+        <v>1</v>
+      </c>
+      <c r="Z9">
+        <v>1</v>
+      </c>
+      <c r="AA9">
+        <v>14</v>
+      </c>
+      <c r="AB9">
+        <v>0</v>
+      </c>
+      <c r="AC9">
+        <v>0</v>
+      </c>
+      <c r="AD9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>08/05/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C10">
+        <v>6830</v>
+      </c>
+      <c r="D10">
+        <v>4350</v>
+      </c>
+      <c r="E10">
+        <v>120</v>
+      </c>
+      <c r="F10">
+        <v>4230</v>
+      </c>
+      <c r="G10">
+        <v>2480</v>
+      </c>
+      <c r="H10">
+        <v>52</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>31</v>
+      </c>
+      <c r="K10">
+        <v>6</v>
+      </c>
+      <c r="L10">
+        <v>20</v>
+      </c>
+      <c r="M10">
+        <v>7</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>116</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>2</v>
+      </c>
+      <c r="U10">
+        <v>7</v>
+      </c>
+      <c r="V10">
+        <v>12</v>
+      </c>
+      <c r="W10">
+        <v>1</v>
+      </c>
+      <c r="X10">
+        <v>1</v>
+      </c>
+      <c r="Y10">
+        <v>1</v>
+      </c>
+      <c r="Z10">
+        <v>1</v>
+      </c>
+      <c r="AA10">
+        <v>14</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
+      <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>09/05/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C11">
+        <v>9680</v>
+      </c>
+      <c r="D11">
+        <v>4350</v>
+      </c>
+      <c r="E11">
+        <v>120</v>
+      </c>
+      <c r="F11">
+        <v>4230</v>
+      </c>
+      <c r="G11">
+        <v>5330</v>
+      </c>
+      <c r="H11">
+        <v>62</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>55</v>
+      </c>
+      <c r="K11">
+        <v>5</v>
+      </c>
+      <c r="L11">
+        <v>38</v>
+      </c>
+      <c r="M11">
+        <v>6</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>166</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>3</v>
+      </c>
+      <c r="U11">
+        <v>13</v>
+      </c>
+      <c r="V11">
+        <v>10</v>
+      </c>
+      <c r="W11">
+        <v>2</v>
+      </c>
+      <c r="X11">
+        <v>2</v>
+      </c>
+      <c r="Y11">
+        <v>1</v>
+      </c>
+      <c r="Z11">
+        <v>2</v>
+      </c>
+      <c r="AA11">
+        <v>12</v>
+      </c>
+      <c r="AB11">
+        <v>0</v>
+      </c>
+      <c r="AC11">
+        <v>0</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B13" t="str">
+        <v>9 days</v>
+      </c>
+      <c r="C13">
+        <v>92250</v>
+      </c>
+      <c r="D13">
+        <v>52800</v>
+      </c>
+      <c r="E13">
+        <v>1380</v>
+      </c>
+      <c r="F13">
+        <v>51420</v>
+      </c>
+      <c r="G13">
+        <v>39450</v>
+      </c>
+      <c r="H13">
+        <v>497</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>546</v>
+      </c>
+      <c r="K13">
+        <v>49</v>
+      </c>
+      <c r="L13">
+        <v>404</v>
+      </c>
+      <c r="M13">
+        <v>101</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>1597</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>22</v>
+      </c>
+      <c r="U13">
+        <v>141</v>
+      </c>
+      <c r="V13">
+        <v>98</v>
+      </c>
+      <c r="W13">
+        <v>22</v>
+      </c>
+      <c r="X13">
+        <v>22</v>
+      </c>
+      <c r="Y13">
+        <v>12</v>
+      </c>
+      <c r="Z13">
+        <v>23</v>
+      </c>
+      <c r="AA13">
+        <v>202</v>
+      </c>
+      <c r="AB13">
+        <v>0</v>
+      </c>
+      <c r="AC13">
+        <v>0</v>
+      </c>
+      <c r="AD13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>AVG/DAY</v>
+      </c>
+      <c r="C14">
+        <v>10250</v>
+      </c>
+      <c r="D14">
+        <v>5866.666666666667</v>
+      </c>
+      <c r="E14">
+        <v>153.33333333333334</v>
+      </c>
+      <c r="F14">
+        <v>5713.333333333333</v>
+      </c>
+      <c r="G14">
+        <v>4383.333333333333</v>
+      </c>
+      <c r="H14">
+        <v>55.22222222222222</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>60.666666666666664</v>
+      </c>
+      <c r="K14">
+        <v>5.444444444444445</v>
+      </c>
+      <c r="L14">
+        <v>44.888888888888886</v>
+      </c>
+      <c r="M14">
+        <v>11.222222222222221</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>177.44444444444446</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>2.4444444444444446</v>
+      </c>
+      <c r="U14">
+        <v>15.666666666666666</v>
+      </c>
+      <c r="V14">
+        <v>10.88888888888889</v>
+      </c>
+      <c r="W14">
+        <v>2.4444444444444446</v>
+      </c>
+      <c r="X14">
+        <v>2.4444444444444446</v>
+      </c>
+      <c r="Y14">
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="Z14">
+        <v>2.5555555555555554</v>
+      </c>
+      <c r="AA14">
+        <v>22.444444444444443</v>
+      </c>
+      <c r="AB14">
+        <v>0</v>
+      </c>
+      <c r="AC14">
+        <v>0</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: upgrade to Turbo-Boost AI OCR with Gemini 3.1 & fix May data integrity
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -13749,7 +13749,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD14"/>
+  <dimension ref="A1:AD16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -13856,19 +13856,19 @@
         <v>Fri</v>
       </c>
       <c r="C3">
-        <v>13950</v>
+        <v>13770</v>
       </c>
       <c r="D3">
-        <v>8220</v>
+        <v>8040</v>
       </c>
       <c r="E3">
-        <v>180</v>
+        <v>120</v>
       </c>
       <c r="F3">
-        <v>8040</v>
+        <v>7920</v>
       </c>
       <c r="G3">
-        <v>5730</v>
+        <v>5910</v>
       </c>
       <c r="H3">
         <v>81</v>
@@ -13963,13 +13963,13 @@
         <v>7290</v>
       </c>
       <c r="H4">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="I4">
         <v>0</v>
       </c>
       <c r="J4">
-        <v>126</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>7</v>
@@ -13990,7 +13990,7 @@
         <v>0</v>
       </c>
       <c r="Q4">
-        <v>302</v>
+        <v>92</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -14020,7 +14020,7 @@
         <v>5</v>
       </c>
       <c r="AA4">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="AB4">
         <v>0</v>
@@ -14055,49 +14055,49 @@
         <v>5010</v>
       </c>
       <c r="H5">
+        <v>65</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>88</v>
+      </c>
+      <c r="K5">
+        <v>15</v>
+      </c>
+      <c r="L5">
+        <v>75</v>
+      </c>
+      <c r="M5">
+        <v>39</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>282</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
         <v>63</v>
       </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
+      <c r="U5">
         <v>70</v>
       </c>
-      <c r="K5">
+      <c r="V5">
         <v>5</v>
-      </c>
-      <c r="L5">
-        <v>67</v>
-      </c>
-      <c r="M5">
-        <v>13</v>
-      </c>
-      <c r="N5">
-        <v>0</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <v>218</v>
-      </c>
-      <c r="R5">
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-      <c r="T5">
-        <v>2</v>
-      </c>
-      <c r="U5">
-        <v>18</v>
-      </c>
-      <c r="V5">
-        <v>10</v>
       </c>
       <c r="W5">
         <v>4</v>
@@ -14112,7 +14112,7 @@
         <v>4</v>
       </c>
       <c r="AA5">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="AB5">
         <v>0</v>
@@ -14239,19 +14239,19 @@
         <v>3520</v>
       </c>
       <c r="H7">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L7">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="M7">
         <v>9</v>
@@ -14266,7 +14266,7 @@
         <v>0</v>
       </c>
       <c r="Q7">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="R7">
         <v>0</v>
@@ -14278,10 +14278,10 @@
         <v>1.5</v>
       </c>
       <c r="U7">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="V7">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W7">
         <v>2</v>
@@ -14515,16 +14515,16 @@
         <v>2480</v>
       </c>
       <c r="H10">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K10">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="L10">
         <v>20</v>
@@ -14542,7 +14542,7 @@
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="R10">
         <v>0</v>
@@ -14607,22 +14607,22 @@
         <v>5330</v>
       </c>
       <c r="H11">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="K11">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L11">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="M11">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -14634,7 +14634,7 @@
         <v>0</v>
       </c>
       <c r="Q11">
-        <v>166</v>
+        <v>0</v>
       </c>
       <c r="R11">
         <v>0</v>
@@ -14676,45 +14676,137 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>10/05/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C12">
+        <v>10690</v>
+      </c>
+      <c r="D12">
+        <v>6590</v>
+      </c>
+      <c r="E12">
+        <v>180</v>
+      </c>
+      <c r="F12">
+        <v>6410</v>
+      </c>
+      <c r="G12">
+        <v>4100</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>45</v>
+      </c>
+      <c r="U12">
+        <v>56</v>
+      </c>
+      <c r="V12">
+        <v>9</v>
+      </c>
+      <c r="W12">
+        <v>3</v>
+      </c>
+      <c r="X12">
+        <v>3</v>
+      </c>
+      <c r="Y12">
+        <v>1.5</v>
+      </c>
+      <c r="Z12">
+        <v>3</v>
+      </c>
+      <c r="AA12">
+        <v>9</v>
+      </c>
+      <c r="AB12">
+        <v>0</v>
+      </c>
+      <c r="AC12">
+        <v>0</v>
+      </c>
+      <c r="AD12">
+        <v>0</v>
+      </c>
+    </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>TOTAL</v>
+        <v>11/05/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>9 days</v>
+        <v>Mon</v>
       </c>
       <c r="C13">
-        <v>92250</v>
+        <v>6455</v>
       </c>
       <c r="D13">
-        <v>52800</v>
+        <v>3660</v>
       </c>
       <c r="E13">
-        <v>1380</v>
+        <v>120</v>
       </c>
       <c r="F13">
-        <v>51420</v>
+        <v>3540</v>
       </c>
       <c r="G13">
-        <v>39450</v>
+        <v>2795</v>
       </c>
       <c r="H13">
-        <v>497</v>
+        <v>0</v>
       </c>
       <c r="I13">
         <v>0</v>
       </c>
       <c r="J13">
-        <v>546</v>
+        <v>0</v>
       </c>
       <c r="K13">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="L13">
-        <v>404</v>
+        <v>0</v>
       </c>
       <c r="M13">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="N13">
         <v>0</v>
@@ -14726,7 +14818,7 @@
         <v>0</v>
       </c>
       <c r="Q13">
-        <v>1597</v>
+        <v>0</v>
       </c>
       <c r="R13">
         <v>0</v>
@@ -14735,28 +14827,28 @@
         <v>0</v>
       </c>
       <c r="T13">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="U13">
-        <v>141</v>
+        <v>48</v>
       </c>
       <c r="V13">
-        <v>98</v>
+        <v>3</v>
       </c>
       <c r="W13">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="X13">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="Y13">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="Z13">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="AA13">
-        <v>202</v>
+        <v>7</v>
       </c>
       <c r="AB13">
         <v>0</v>
@@ -14770,40 +14862,43 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>AVG/DAY</v>
+        <v>12/05/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Tue</v>
       </c>
       <c r="C14">
-        <v>10250</v>
+        <v>4770</v>
       </c>
       <c r="D14">
-        <v>5866.666666666667</v>
+        <v>3110</v>
       </c>
       <c r="E14">
-        <v>153.33333333333334</v>
+        <v>120</v>
       </c>
       <c r="F14">
-        <v>5713.333333333333</v>
+        <v>2990</v>
       </c>
       <c r="G14">
-        <v>4383.333333333333</v>
+        <v>1660</v>
       </c>
       <c r="H14">
-        <v>55.22222222222222</v>
+        <v>0</v>
       </c>
       <c r="I14">
         <v>0</v>
       </c>
       <c r="J14">
-        <v>60.666666666666664</v>
+        <v>0</v>
       </c>
       <c r="K14">
-        <v>5.444444444444445</v>
+        <v>3</v>
       </c>
       <c r="L14">
-        <v>44.888888888888886</v>
+        <v>26</v>
       </c>
       <c r="M14">
-        <v>11.222222222222221</v>
+        <v>9</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -14815,7 +14910,7 @@
         <v>0</v>
       </c>
       <c r="Q14">
-        <v>177.44444444444446</v>
+        <v>38</v>
       </c>
       <c r="R14">
         <v>0</v>
@@ -14824,28 +14919,28 @@
         <v>0</v>
       </c>
       <c r="T14">
-        <v>2.4444444444444446</v>
+        <v>6</v>
       </c>
       <c r="U14">
-        <v>15.666666666666666</v>
+        <v>6</v>
       </c>
       <c r="V14">
-        <v>10.88888888888889</v>
+        <v>6</v>
       </c>
       <c r="W14">
-        <v>2.4444444444444446</v>
+        <v>0</v>
       </c>
       <c r="X14">
-        <v>2.4444444444444446</v>
+        <v>2</v>
       </c>
       <c r="Y14">
-        <v>1.3333333333333333</v>
+        <v>1</v>
       </c>
       <c r="Z14">
-        <v>2.5555555555555554</v>
+        <v>1</v>
       </c>
       <c r="AA14">
-        <v>22.444444444444443</v>
+        <v>18</v>
       </c>
       <c r="AB14">
         <v>0</v>
@@ -14854,12 +14949,196 @@
         <v>0</v>
       </c>
       <c r="AD14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>13/05/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C15">
+        <v>9380</v>
+      </c>
+      <c r="D15">
+        <v>5350</v>
+      </c>
+      <c r="E15">
+        <v>150</v>
+      </c>
+      <c r="F15">
+        <v>5200</v>
+      </c>
+      <c r="G15">
+        <v>4030</v>
+      </c>
+      <c r="H15">
+        <v>55</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>43</v>
+      </c>
+      <c r="K15">
+        <v>5</v>
+      </c>
+      <c r="L15">
+        <v>46</v>
+      </c>
+      <c r="M15">
+        <v>12</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>161</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>2</v>
+      </c>
+      <c r="U15">
+        <v>12</v>
+      </c>
+      <c r="V15">
+        <v>10</v>
+      </c>
+      <c r="W15">
+        <v>3</v>
+      </c>
+      <c r="X15">
+        <v>3</v>
+      </c>
+      <c r="Y15">
+        <v>1</v>
+      </c>
+      <c r="Z15">
+        <v>2</v>
+      </c>
+      <c r="AA15">
+        <v>24</v>
+      </c>
+      <c r="AB15">
+        <v>0</v>
+      </c>
+      <c r="AC15">
+        <v>0</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>14/05/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C16">
+        <v>7890</v>
+      </c>
+      <c r="D16">
+        <v>4330</v>
+      </c>
+      <c r="E16">
+        <v>120</v>
+      </c>
+      <c r="F16">
+        <v>4210</v>
+      </c>
+      <c r="G16">
+        <v>3560</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>2.5</v>
+      </c>
+      <c r="U16">
+        <v>9</v>
+      </c>
+      <c r="V16">
+        <v>5</v>
+      </c>
+      <c r="W16">
+        <v>2</v>
+      </c>
+      <c r="X16">
+        <v>2</v>
+      </c>
+      <c r="Y16">
+        <v>1</v>
+      </c>
+      <c r="Z16">
+        <v>2</v>
+      </c>
+      <c r="AA16">
+        <v>30</v>
+      </c>
+      <c r="AB16">
+        <v>0</v>
+      </c>
+      <c r="AC16">
+        <v>0</v>
+      </c>
+      <c r="AD16">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(dashboard): resolve mobile view crash in private browsing and host script dependencies locally
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F288"/>
+  <dimension ref="A1:F304"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6895,9 +6895,329 @@
         <v>50</v>
       </c>
     </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>15/06/2026</v>
+      </c>
+      <c r="B289" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C289" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D289" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="E289" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="F289">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>15/06/2026</v>
+      </c>
+      <c r="B290" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C290" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D290" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="E290" t="str">
+        <v>สับปะรด 12 ลูก</v>
+      </c>
+      <c r="F290">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>15/06/2026</v>
+      </c>
+      <c r="B291" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C291" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D291" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="E291" t="str">
+        <v>ฝรั่ง 1 ตะกร้า</v>
+      </c>
+      <c r="F291">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>17/06/2026</v>
+      </c>
+      <c r="B292" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C292" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D292" t="str">
+        <v>Orange</v>
+      </c>
+      <c r="E292" t="str">
+        <v>รอบ 09/06/69</v>
+      </c>
+      <c r="F292">
+        <v>16445</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>18/06/2026</v>
+      </c>
+      <c r="B293" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C293" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D293" t="str">
+        <v>Mango</v>
+      </c>
+      <c r="E293" t="str">
+        <v>มะม่วง 1 ลัง</v>
+      </c>
+      <c r="F293">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>18/06/2026</v>
+      </c>
+      <c r="B294" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C294" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D294" t="str">
+        <v>Coconut Water</v>
+      </c>
+      <c r="E294" t="str">
+        <v>เนื้อมะพร้าว 20 * 120 2400 น้ำมะพร้าว 20 *</v>
+      </c>
+      <c r="F294">
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>18/06/2026</v>
+      </c>
+      <c r="B295" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C295" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D295" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="E295" t="str">
+        <v>ฝรั่ง 1 ตะกร้า</v>
+      </c>
+      <c r="F295">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>19/06/2026</v>
+      </c>
+      <c r="B296" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C296" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D296" t="str">
+        <v>Coconut Water</v>
+      </c>
+      <c r="E296" t="str">
+        <v>น้ำมะพร้าว40ลิตร ลิตรละ45บาท</v>
+      </c>
+      <c r="F296">
+        <v>5700</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>19/06/2026</v>
+      </c>
+      <c r="B297" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C297" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D297" t="str">
+        <v>Packaging</v>
+      </c>
+      <c r="E297" t="str">
+        <v>น้ำยาล้างจาน 7 ถุง ผงซักฟอก 1</v>
+      </c>
+      <c r="F297">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>21/06/2026</v>
+      </c>
+      <c r="B298" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C298" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D298" t="str">
+        <v>Watermelon</v>
+      </c>
+      <c r="E298" t="str">
+        <v>15-6-2569 แตงโม 50บาท 50 ลูก ยอด 2,500</v>
+      </c>
+      <c r="F298">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>22/06/2026</v>
+      </c>
+      <c r="B299" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C299" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D299" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="E299" t="str">
+        <v>สับปะรด 15 ลูก</v>
+      </c>
+      <c r="F299">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>22/06/2026</v>
+      </c>
+      <c r="B300" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C300" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D300" t="str">
+        <v>Mango</v>
+      </c>
+      <c r="E300" t="str">
+        <v>มะม่วง 2 ลัง</v>
+      </c>
+      <c r="F300">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>22/06/2026</v>
+      </c>
+      <c r="B301" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C301" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D301" t="str">
+        <v>Transportation</v>
+      </c>
+      <c r="E301" t="str">
+        <v>Lalamove</v>
+      </c>
+      <c r="F301">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>22/06/2026</v>
+      </c>
+      <c r="B302" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C302" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D302" t="str">
+        <v>Apple</v>
+      </c>
+      <c r="E302" t="str">
+        <v>แอพเปิ้ล 5 ลัง</v>
+      </c>
+      <c r="F302">
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>22/06/2026</v>
+      </c>
+      <c r="B303" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C303" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D303" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="E303" t="str">
+        <v>สับปะรด 15 ลูก</v>
+      </c>
+      <c r="F303">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>22/06/2026</v>
+      </c>
+      <c r="B304" t="str">
+        <v>Jun26</v>
+      </c>
+      <c r="C304" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D304" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="E304" t="str">
+        <v>ฝรั่ง 1 ลัง</v>
+      </c>
+      <c r="F304">
+        <v>700</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F288"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F304"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -18671,22 +18991,22 @@
         <v>107890</v>
       </c>
       <c r="H34">
-        <v>1379</v>
+        <v>1468</v>
       </c>
       <c r="I34">
         <v>0</v>
       </c>
       <c r="J34">
-        <v>1263</v>
+        <v>1383</v>
       </c>
       <c r="K34">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="L34">
-        <v>1000</v>
+        <v>988</v>
       </c>
       <c r="M34">
-        <v>292</v>
+        <v>306</v>
       </c>
       <c r="N34">
         <v>0</v>
@@ -18698,7 +19018,7 @@
         <v>0</v>
       </c>
       <c r="Q34">
-        <v>4068</v>
+        <v>4286</v>
       </c>
       <c r="R34">
         <v>0</v>
@@ -18760,22 +19080,22 @@
         <v>3596.3333333333335</v>
       </c>
       <c r="H35">
-        <v>45.96666666666667</v>
+        <v>48.93333333333333</v>
       </c>
       <c r="I35">
         <v>0</v>
       </c>
       <c r="J35">
-        <v>42.1</v>
+        <v>46.1</v>
       </c>
       <c r="K35">
-        <v>4.466666666666667</v>
+        <v>4.7</v>
       </c>
       <c r="L35">
-        <v>33.333333333333336</v>
+        <v>32.93333333333333</v>
       </c>
       <c r="M35">
-        <v>9.733333333333333</v>
+        <v>10.2</v>
       </c>
       <c r="N35">
         <v>0</v>
@@ -18787,7 +19107,7 @@
         <v>0</v>
       </c>
       <c r="Q35">
-        <v>135.6</v>
+        <v>142.86666666666667</v>
       </c>
       <c r="R35">
         <v>0</v>
@@ -18838,7 +19158,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD19"/>
+  <dimension ref="A1:AD25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20225,45 +20545,137 @@
         <v>0</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>15/06/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C17">
+        <v>7080</v>
+      </c>
+      <c r="D17">
+        <v>4290</v>
+      </c>
+      <c r="E17">
+        <v>120</v>
+      </c>
+      <c r="F17">
+        <v>4170</v>
+      </c>
+      <c r="G17">
+        <v>2790</v>
+      </c>
+      <c r="H17">
+        <v>34</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>63</v>
+      </c>
+      <c r="K17">
+        <v>5</v>
+      </c>
+      <c r="L17">
+        <v>16</v>
+      </c>
+      <c r="M17">
+        <v>8</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>126</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <v>1.5</v>
+      </c>
+      <c r="U17">
+        <v>12</v>
+      </c>
+      <c r="V17">
+        <v>10</v>
+      </c>
+      <c r="W17">
+        <v>2</v>
+      </c>
+      <c r="X17">
+        <v>2</v>
+      </c>
+      <c r="Y17">
+        <v>1</v>
+      </c>
+      <c r="Z17">
+        <v>2</v>
+      </c>
+      <c r="AA17">
+        <v>16</v>
+      </c>
+      <c r="AB17">
+        <v>0</v>
+      </c>
+      <c r="AC17">
+        <v>0</v>
+      </c>
+      <c r="AD17">
+        <v>0</v>
+      </c>
+    </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>TOTAL</v>
+        <v>16/06/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>13 days</v>
+        <v>Tue</v>
       </c>
       <c r="C18">
-        <v>78440</v>
+        <v>4190</v>
       </c>
       <c r="D18">
-        <v>43390</v>
+        <v>1200</v>
       </c>
       <c r="E18">
-        <v>1540</v>
+        <v>60</v>
       </c>
       <c r="F18">
-        <v>41850</v>
+        <v>1140</v>
       </c>
       <c r="G18">
-        <v>35050</v>
+        <v>2990</v>
       </c>
       <c r="H18">
-        <v>419</v>
+        <v>24</v>
       </c>
       <c r="I18">
         <v>0</v>
       </c>
       <c r="J18">
-        <v>319</v>
+        <v>40</v>
       </c>
       <c r="K18">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="L18">
-        <v>233</v>
+        <v>5</v>
       </c>
       <c r="M18">
-        <v>141</v>
+        <v>5</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -20275,7 +20687,7 @@
         <v>0</v>
       </c>
       <c r="Q18">
-        <v>1163</v>
+        <v>75</v>
       </c>
       <c r="R18">
         <v>0</v>
@@ -20284,28 +20696,28 @@
         <v>0</v>
       </c>
       <c r="T18">
-        <v>103.2</v>
+        <v>1</v>
       </c>
       <c r="U18">
-        <v>119.4</v>
+        <v>8</v>
       </c>
       <c r="V18">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="W18">
-        <v>18.5</v>
+        <v>1</v>
       </c>
       <c r="X18">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="Y18">
-        <v>10.5</v>
+        <v>0</v>
       </c>
       <c r="Z18">
+        <v>1</v>
+      </c>
+      <c r="AA18">
         <v>10</v>
-      </c>
-      <c r="AA18">
-        <v>209</v>
       </c>
       <c r="AB18">
         <v>0</v>
@@ -20319,96 +20731,556 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>17/06/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C19">
+        <v>8450</v>
+      </c>
+      <c r="D19">
+        <v>5530</v>
+      </c>
+      <c r="E19">
+        <v>120</v>
+      </c>
+      <c r="F19">
+        <v>5410</v>
+      </c>
+      <c r="G19">
+        <v>2920</v>
+      </c>
+      <c r="H19">
+        <v>47</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>52</v>
+      </c>
+      <c r="K19">
+        <v>11</v>
+      </c>
+      <c r="L19">
+        <v>27</v>
+      </c>
+      <c r="M19">
+        <v>17</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>154</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>2</v>
+      </c>
+      <c r="U19">
+        <v>10</v>
+      </c>
+      <c r="V19">
+        <v>22</v>
+      </c>
+      <c r="W19">
+        <v>3</v>
+      </c>
+      <c r="X19">
+        <v>3</v>
+      </c>
+      <c r="Y19">
+        <v>1</v>
+      </c>
+      <c r="Z19">
+        <v>3</v>
+      </c>
+      <c r="AA19">
+        <v>34</v>
+      </c>
+      <c r="AB19">
+        <v>0</v>
+      </c>
+      <c r="AC19">
+        <v>0</v>
+      </c>
+      <c r="AD19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>18/06/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C20">
+        <v>4960</v>
+      </c>
+      <c r="D20">
+        <v>3960</v>
+      </c>
+      <c r="E20">
+        <v>90</v>
+      </c>
+      <c r="F20">
+        <v>3870</v>
+      </c>
+      <c r="G20">
+        <v>1000</v>
+      </c>
+      <c r="H20">
+        <v>17</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>53</v>
+      </c>
+      <c r="K20">
+        <v>3</v>
+      </c>
+      <c r="L20">
+        <v>6</v>
+      </c>
+      <c r="M20">
+        <v>8</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>87</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20">
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <v>1</v>
+      </c>
+      <c r="U20">
+        <v>9</v>
+      </c>
+      <c r="V20">
+        <v>6</v>
+      </c>
+      <c r="W20">
+        <v>1</v>
+      </c>
+      <c r="X20">
+        <v>1</v>
+      </c>
+      <c r="Y20">
+        <v>0</v>
+      </c>
+      <c r="Z20">
+        <v>1</v>
+      </c>
+      <c r="AA20">
+        <v>16</v>
+      </c>
+      <c r="AB20">
+        <v>0</v>
+      </c>
+      <c r="AC20">
+        <v>0</v>
+      </c>
+      <c r="AD20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>19/06/2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C21">
+        <v>2880</v>
+      </c>
+      <c r="D21">
+        <v>840</v>
+      </c>
+      <c r="E21">
+        <v>60</v>
+      </c>
+      <c r="F21">
+        <v>780</v>
+      </c>
+      <c r="G21">
+        <v>2040</v>
+      </c>
+      <c r="H21">
+        <v>12</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>21</v>
+      </c>
+      <c r="K21">
+        <v>5</v>
+      </c>
+      <c r="L21">
+        <v>7</v>
+      </c>
+      <c r="M21">
+        <v>2</v>
+      </c>
+      <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21">
+        <v>47</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <v>1</v>
+      </c>
+      <c r="U21">
+        <v>5</v>
+      </c>
+      <c r="V21">
+        <v>10</v>
+      </c>
+      <c r="W21">
+        <v>1.5</v>
+      </c>
+      <c r="X21">
+        <v>1</v>
+      </c>
+      <c r="Y21">
+        <v>0</v>
+      </c>
+      <c r="Z21">
+        <v>1</v>
+      </c>
+      <c r="AA21">
+        <v>4</v>
+      </c>
+      <c r="AB21">
+        <v>0</v>
+      </c>
+      <c r="AC21">
+        <v>0</v>
+      </c>
+      <c r="AD21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>20/06/2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C22">
+        <v>11630</v>
+      </c>
+      <c r="D22">
+        <v>6190</v>
+      </c>
+      <c r="E22">
+        <v>180</v>
+      </c>
+      <c r="F22">
+        <v>6010</v>
+      </c>
+      <c r="G22">
+        <v>5440</v>
+      </c>
+      <c r="H22">
+        <v>63</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>79</v>
+      </c>
+      <c r="K22">
+        <v>19</v>
+      </c>
+      <c r="L22">
+        <v>31</v>
+      </c>
+      <c r="M22">
+        <v>16</v>
+      </c>
+      <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22">
+        <v>208</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
+        <v>0</v>
+      </c>
+      <c r="T22">
+        <v>2.5</v>
+      </c>
+      <c r="U22">
+        <v>12</v>
+      </c>
+      <c r="V22">
+        <v>38</v>
+      </c>
+      <c r="W22">
+        <v>4</v>
+      </c>
+      <c r="X22">
+        <v>4</v>
+      </c>
+      <c r="Y22">
+        <v>1</v>
+      </c>
+      <c r="Z22">
+        <v>4</v>
+      </c>
+      <c r="AA22">
+        <v>32</v>
+      </c>
+      <c r="AB22">
+        <v>0</v>
+      </c>
+      <c r="AC22">
+        <v>0</v>
+      </c>
+      <c r="AD22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B24" t="str">
+        <v>20 days</v>
+      </c>
+      <c r="C24">
+        <v>124150</v>
+      </c>
+      <c r="D24">
+        <v>67420</v>
+      </c>
+      <c r="E24">
+        <v>2290</v>
+      </c>
+      <c r="F24">
+        <v>65130</v>
+      </c>
+      <c r="G24">
+        <v>56730</v>
+      </c>
+      <c r="H24">
+        <v>731</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>779</v>
+      </c>
+      <c r="K24">
+        <v>96</v>
+      </c>
+      <c r="L24">
+        <v>339</v>
+      </c>
+      <c r="M24">
+        <v>205</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24">
+        <v>2150</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>8</v>
+      </c>
+      <c r="T24">
+        <v>32.5</v>
+      </c>
+      <c r="U24">
+        <v>150</v>
+      </c>
+      <c r="V24">
+        <v>148</v>
+      </c>
+      <c r="W24">
+        <v>32.5</v>
+      </c>
+      <c r="X24">
+        <v>32.5</v>
+      </c>
+      <c r="Y24">
+        <v>14.5</v>
+      </c>
+      <c r="Z24">
+        <v>23</v>
+      </c>
+      <c r="AA24">
+        <v>347</v>
+      </c>
+      <c r="AB24">
+        <v>0</v>
+      </c>
+      <c r="AC24">
+        <v>0</v>
+      </c>
+      <c r="AD24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
         <v>AVG/DAY</v>
       </c>
-      <c r="C19">
-        <v>6033.846153846154</v>
-      </c>
-      <c r="D19">
-        <v>3337.6923076923076</v>
-      </c>
-      <c r="E19">
-        <v>118.46153846153847</v>
-      </c>
-      <c r="F19">
-        <v>3219.230769230769</v>
-      </c>
-      <c r="G19">
-        <v>2696.153846153846</v>
-      </c>
-      <c r="H19">
-        <v>32.23076923076923</v>
-      </c>
-      <c r="I19">
-        <v>0</v>
-      </c>
-      <c r="J19">
-        <v>24.53846153846154</v>
-      </c>
-      <c r="K19">
-        <v>3.923076923076923</v>
-      </c>
-      <c r="L19">
-        <v>17.923076923076923</v>
-      </c>
-      <c r="M19">
-        <v>10.846153846153847</v>
-      </c>
-      <c r="N19">
-        <v>0</v>
-      </c>
-      <c r="O19">
-        <v>0</v>
-      </c>
-      <c r="P19">
-        <v>0</v>
-      </c>
-      <c r="Q19">
-        <v>89.46153846153847</v>
-      </c>
-      <c r="R19">
-        <v>0</v>
-      </c>
-      <c r="S19">
-        <v>0</v>
-      </c>
-      <c r="T19">
-        <v>7.938461538461539</v>
-      </c>
-      <c r="U19">
-        <v>9.184615384615386</v>
-      </c>
-      <c r="V19">
-        <v>4.461538461538462</v>
-      </c>
-      <c r="W19">
-        <v>1.4230769230769231</v>
-      </c>
-      <c r="X19">
-        <v>1.4615384615384615</v>
-      </c>
-      <c r="Y19">
-        <v>0.8076923076923077</v>
-      </c>
-      <c r="Z19">
-        <v>0.7692307692307693</v>
-      </c>
-      <c r="AA19">
-        <v>16.076923076923077</v>
-      </c>
-      <c r="AB19">
-        <v>0</v>
-      </c>
-      <c r="AC19">
-        <v>0</v>
-      </c>
-      <c r="AD19">
+      <c r="C25">
+        <v>6207.5</v>
+      </c>
+      <c r="D25">
+        <v>3371</v>
+      </c>
+      <c r="E25">
+        <v>114.5</v>
+      </c>
+      <c r="F25">
+        <v>3256.5</v>
+      </c>
+      <c r="G25">
+        <v>2836.5</v>
+      </c>
+      <c r="H25">
+        <v>36.55</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>38.95</v>
+      </c>
+      <c r="K25">
+        <v>4.8</v>
+      </c>
+      <c r="L25">
+        <v>16.95</v>
+      </c>
+      <c r="M25">
+        <v>10.25</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25">
+        <v>107.5</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25">
+        <v>0.4</v>
+      </c>
+      <c r="T25">
+        <v>1.625</v>
+      </c>
+      <c r="U25">
+        <v>7.5</v>
+      </c>
+      <c r="V25">
+        <v>7.4</v>
+      </c>
+      <c r="W25">
+        <v>1.625</v>
+      </c>
+      <c r="X25">
+        <v>1.625</v>
+      </c>
+      <c r="Y25">
+        <v>0.725</v>
+      </c>
+      <c r="Z25">
+        <v>1.15</v>
+      </c>
+      <c r="AA25">
+        <v>17.35</v>
+      </c>
+      <c r="AB25">
+        <v>0</v>
+      </c>
+      <c r="AC25">
+        <v>0</v>
+      </c>
+      <c r="AD25">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: correct COGS/OPEX/CAPEX miscategorization across Jan-Jun26 expenses
Audited all B1/B2 expense slips against categorize() rules and applied 34
corrections: reclassified generic Stock purchases from OPEX/Investment to
COGS/Stock, fixed a legacy "Ice" mis-tag on ~24 unrelated entries (tolls,
medical bills, electricity, hardware), moved 4 misfiled watermelon/apple/
pineapple purchases from OPEX to COGS, fixed a cold-press machine and
mangosteen entry, zeroed a duplicate pineapple charge, and excluded two
Jan26 partner profit-share payouts (~78k) that were incorrectly booked as
COGS/Ice expenses instead of post-profit distributions. Documented the
categorization pitfalls in CLAUDE.md/GEMINI.md/AGENTS.md for future agents.
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -1263,16 +1263,16 @@
         <v>Jan26</v>
       </c>
       <c r="C7" t="str">
-        <v>COGS</v>
+        <v>EXCLUDED</v>
       </c>
       <c r="D7" t="str">
-        <v>Ice</v>
+        <v>Profit Distribution</v>
       </c>
       <c r="E7" t="str">
-        <v>ส่วนแบ่ง60เปอ</v>
+        <v>ส่วนแบ่ง60เปอ — removed from P&amp;L, this is a partner profit-share payout, not a business expense (owner-confirmed)</v>
       </c>
       <c r="F7">
-        <v>47961</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1283,16 +1283,16 @@
         <v>Jan26</v>
       </c>
       <c r="C8" t="str">
-        <v>COGS</v>
+        <v>EXCLUDED</v>
       </c>
       <c r="D8" t="str">
-        <v>Ice</v>
+        <v>Profit Distribution</v>
       </c>
       <c r="E8" t="str">
-        <v>ค่าส่วนแบ่งกำไรเมน 40เปอ</v>
+        <v>ค่าส่วนแบ่งกำไรเมน 40เปอ — removed from P&amp;L, this is a partner profit-share payout, not a business expense (owner-confirmed)</v>
       </c>
       <c r="F8">
-        <v>32000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1486,7 +1486,7 @@
         <v>COGS</v>
       </c>
       <c r="D18" t="str">
-        <v>Ice</v>
+        <v>Transportation</v>
       </c>
       <c r="E18" t="str">
         <v>ค่าขนตะกร้ากลับ</v>
@@ -2343,10 +2343,10 @@
         <v>Feb26</v>
       </c>
       <c r="C61" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D61" t="str">
-        <v>Ice</v>
+        <v>Fixed Costs</v>
       </c>
       <c r="E61" t="str">
         <v>ค่าไฟเดือนมค</v>
@@ -2383,10 +2383,10 @@
         <v>Feb26</v>
       </c>
       <c r="C63" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D63" t="str">
-        <v>Other</v>
+        <v>Watermelon</v>
       </c>
       <c r="E63" t="str">
         <v>Unknown</v>
@@ -2406,7 +2406,7 @@
         <v>COGS</v>
       </c>
       <c r="D64" t="str">
-        <v>Ice</v>
+        <v>Apple</v>
       </c>
       <c r="E64" t="str">
         <v>Unknown</v>
@@ -2543,10 +2543,10 @@
         <v>Feb26</v>
       </c>
       <c r="C71" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D71" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E71" t="str">
         <v>ผ้าปิดร้าน 218 ค่ารถ 198</v>
@@ -2923,10 +2923,10 @@
         <v>Mar26</v>
       </c>
       <c r="C90" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D90" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E90" t="str">
         <v>ค่าทางด่วน</v>
@@ -3163,10 +3163,10 @@
         <v>Mar26</v>
       </c>
       <c r="C102" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D102" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E102" t="str">
         <v>ค่าทางด่วน</v>
@@ -3203,10 +3203,10 @@
         <v>Mar26</v>
       </c>
       <c r="C104" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D104" t="str">
-        <v>Ice</v>
+        <v>Fixed Costs</v>
       </c>
       <c r="E104" t="str">
         <v>ค่าไฟเดือนกพ มีนา</v>
@@ -3243,10 +3243,10 @@
         <v>Mar26</v>
       </c>
       <c r="C106" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D106" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E106" t="str">
         <v>สกรู กาวตะปู</v>
@@ -3303,10 +3303,10 @@
         <v>Mar26</v>
       </c>
       <c r="C109" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D109" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E109" t="str">
         <v>รถเข็นของคันใหม่</v>
@@ -3626,7 +3626,7 @@
         <v>COGS</v>
       </c>
       <c r="D125" t="str">
-        <v>Ice</v>
+        <v>Water</v>
       </c>
       <c r="E125" t="str">
         <v>เนื้อ 1200 น้ำ 500</v>
@@ -3786,7 +3786,7 @@
         <v>COGS</v>
       </c>
       <c r="D133" t="str">
-        <v>Ice</v>
+        <v>Milk/Conden</v>
       </c>
       <c r="E133" t="str">
         <v>ค่านม</v>
@@ -3846,7 +3846,7 @@
         <v>COGS</v>
       </c>
       <c r="D136" t="str">
-        <v>Ice</v>
+        <v>Water</v>
       </c>
       <c r="E136" t="str">
         <v>น้ำ 500 เนื้อ 1200</v>
@@ -4246,7 +4246,7 @@
         <v>COGS</v>
       </c>
       <c r="D156" t="str">
-        <v>Ice</v>
+        <v>Water</v>
       </c>
       <c r="E156" t="str">
         <v>16/4/26 เนื้อ 10 น้ำ 10 21/4/26 เนื้อ 10</v>
@@ -4626,7 +4626,7 @@
         <v>COGS</v>
       </c>
       <c r="D175" t="str">
-        <v>Ice</v>
+        <v>Pineapple</v>
       </c>
       <c r="E175" t="str">
         <v>สับปะรส 3 ตะกร้า</v>
@@ -4686,7 +4686,7 @@
         <v>OPEX</v>
       </c>
       <c r="D178" t="str">
-        <v>Fixed Costs</v>
+        <v>Rental</v>
       </c>
       <c r="E178" t="str">
         <v>Rent</v>
@@ -4703,10 +4703,10 @@
         <v>Apr26</v>
       </c>
       <c r="C179" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D179" t="str">
-        <v>Investment</v>
+        <v>Stock</v>
       </c>
       <c r="E179" t="str">
         <v>Stock (Allocated 82.9%)</v>
@@ -4729,10 +4729,10 @@
         <v>Other</v>
       </c>
       <c r="E180" t="str">
-        <v>Pineapple</v>
+        <v>Pineapple (duplicate of 30/04/2026 slip entry, zeroed to avoid double-count)</v>
       </c>
       <c r="F180">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181">
@@ -4823,10 +4823,10 @@
         <v>May26</v>
       </c>
       <c r="C185" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D185" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E185" t="str">
         <v>ค่าหาหมอเอ</v>
@@ -4843,10 +4843,10 @@
         <v>May26</v>
       </c>
       <c r="C186" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D186" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E186" t="str">
         <v>ค่าหมอเอ</v>
@@ -4923,10 +4923,10 @@
         <v>May26</v>
       </c>
       <c r="C190" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D190" t="str">
-        <v>Other</v>
+        <v>Watermelon</v>
       </c>
       <c r="E190" t="str">
         <v>30-4-2569 เบอร์ 70฿ 60 ลูก</v>
@@ -5103,10 +5103,10 @@
         <v>May26</v>
       </c>
       <c r="C199" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D199" t="str">
-        <v>Other</v>
+        <v>Watermelon</v>
       </c>
       <c r="E199" t="str">
         <v>4-5-2569 เบอร์ 70฿ 60 ลูก ยอด 4,200</v>
@@ -5383,10 +5383,10 @@
         <v>May26</v>
       </c>
       <c r="C213" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D213" t="str">
-        <v>Other</v>
+        <v>Watermelon</v>
       </c>
       <c r="E213" t="str">
         <v>11-5-2569 50 ลูก ยอด 4,000</v>
@@ -5563,10 +5563,10 @@
         <v>May26</v>
       </c>
       <c r="C222" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D222" t="str">
-        <v>Other</v>
+        <v>Pineapple</v>
       </c>
       <c r="E222" t="str">
         <v>14/05/26 18 ลูก 504 บาท 16/05/26 18 ลูก</v>
@@ -5743,10 +5743,10 @@
         <v>May26</v>
       </c>
       <c r="C231" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D231" t="str">
-        <v>Other</v>
+        <v>Watermelon</v>
       </c>
       <c r="E231" t="str">
         <v>16-5-2569ยอด 4,000฿</v>
@@ -6103,10 +6103,10 @@
         <v>May26</v>
       </c>
       <c r="C249" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D249" t="str">
-        <v>Other</v>
+        <v>Apple</v>
       </c>
       <c r="E249" t="str">
         <v>Unknown</v>
@@ -6143,10 +6143,10 @@
         <v>May26</v>
       </c>
       <c r="C251" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D251" t="str">
-        <v>Investment</v>
+        <v>Stock</v>
       </c>
       <c r="E251" t="str">
         <v>Stock Adjustment (Allocated to B2)</v>
@@ -7203,10 +7203,10 @@
         <v>Jun26</v>
       </c>
       <c r="C304" t="str">
-        <v>OPEX</v>
+        <v>CAPEX</v>
       </c>
       <c r="D304" t="str">
-        <v>Other</v>
+        <v>Investment</v>
       </c>
       <c r="E304" t="str">
         <v>สกัดเย็น1เครื่อง</v>
@@ -7243,7 +7243,7 @@
         <v>Jun26</v>
       </c>
       <c r="C306" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D306" t="str">
         <v>Other</v>

</xml_diff>

<commit_message>
fix: recover missing May26 B1 salary and Mar26 water bill expenses
- May26 B1: filled ฿24,000 salary placeholder (Aye+Wai) that OCR failed
  to parse from the non-standard combined-branch SCB transfer slip.
- Mar26 B1: added the ฿449.25 MWA water bill that was never ingested by
  the OCR pipeline (physical receipt, not a bank transfer slip).
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F319"/>
+  <dimension ref="A1:F320"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6169,10 +6169,10 @@
         <v>Salary</v>
       </c>
       <c r="E252" t="str">
-        <v>Unknown</v>
+        <v>Aye 12,000 + Wai 12,000 (May salary, B1 portion split from joint ฿41,200 SCB transfer 01/06 - see cost_may26.md)</v>
       </c>
       <c r="F252">
-        <v>0</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="253">
@@ -7515,9 +7515,29 @@
         <v>12000</v>
       </c>
     </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>20/03/2026</v>
+      </c>
+      <c r="B320" t="str">
+        <v>Mar26</v>
+      </c>
+      <c r="C320" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D320" t="str">
+        <v>Fixed Costs</v>
+      </c>
+      <c r="E320" t="str">
+        <v>ค่าน้ำประปา เดือน 03/69 (MWA water bill, was never ingested by OCR pipeline)</v>
+      </c>
+      <c r="F320">
+        <v>449.25</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F319"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F320"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: resolve 6 of 17 ambiguous expense entries (Mar-May26)
- Mar26 ฿49,560 unlabeled slip -> Orange (recipient account matches known supplier)
- Apr26 ฿420 barley/red-bean drink mix -> COGS/Other (was Packaging, false keyword match)
- May26 ฿2,820 water+coconut slip -> COGS/Water (was Packaging, "bottle" false match)
- May26 ฿4,875 and ฿2,902 milk-majority slips -> COGS/Milk/Conden (were Packaging)
- May26 ฿1,122 milk+cash-drawer slip split: ฿636 stays COGS/Milk/Conden,
  ฿486 drawer moved to OPEX/Other (equipment, not COGS)

Remaining 11 ambiguous entries are genuinely un-splittable multi-item
purchases or unverifiable low-value slips - left as-is per owner review.
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F320"/>
+  <dimension ref="A1:F321"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3546,7 +3546,7 @@
         <v>COGS</v>
       </c>
       <c r="D121" t="str">
-        <v>Ice</v>
+        <v>Orange</v>
       </c>
       <c r="E121" t="str">
         <v>Unknown</v>
@@ -4286,7 +4286,7 @@
         <v>COGS</v>
       </c>
       <c r="D158" t="str">
-        <v>Packaging</v>
+        <v>Other</v>
       </c>
       <c r="E158" t="str">
         <v>บาร์เลย 4 ถั่วแดง 3 ถุงละ 60</v>
@@ -5066,7 +5066,7 @@
         <v>COGS</v>
       </c>
       <c r="D197" t="str">
-        <v>Packaging</v>
+        <v>Water</v>
       </c>
       <c r="E197" t="str">
         <v>6 พ.ค. น้ำ 30 ขวด 1500 บาท เนื้อ 11 โล 1320 บาท</v>
@@ -5149,10 +5149,10 @@
         <v>Milk/Conden</v>
       </c>
       <c r="E201" t="str">
-        <v>นมข้นจืด 1ลัง 636</v>
+        <v>นมข้นจืด 1ลัง (drawer portion split out below)</v>
       </c>
       <c r="F201">
-        <v>1122</v>
+        <v>636</v>
       </c>
     </row>
     <row r="202">
@@ -5166,7 +5166,7 @@
         <v>COGS</v>
       </c>
       <c r="D202" t="str">
-        <v>Packaging</v>
+        <v>Milk/Conden</v>
       </c>
       <c r="E202" t="str">
         <v>นมข้น 3 ลัง 2568</v>
@@ -5826,7 +5826,7 @@
         <v>COGS</v>
       </c>
       <c r="D235" t="str">
-        <v>Packaging</v>
+        <v>Milk/Conden</v>
       </c>
       <c r="E235" t="str">
         <v>ฝา1 788</v>
@@ -7535,9 +7535,29 @@
         <v>449.25</v>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>09/05/2026</v>
+      </c>
+      <c r="B321" t="str">
+        <v>May26</v>
+      </c>
+      <c r="C321" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D321" t="str">
+        <v>Other</v>
+      </c>
+      <c r="E321" t="str">
+        <v>ลิ้นชักเก็บเงิน (cash register drawer, split from combined 09/05 milk+equipment slip)</v>
+      </c>
+      <c r="F321">
+        <v>486</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F320"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F321"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: resolve remaining ambiguous entries per owner review (Feb-May26)
- Feb26 05/03 duplicate 7,312 orange charge: confirmed already deduped
  by a prior automated pass, no action needed
- Feb26 08/02 798 unlabeled -> OPEX/Other (owner: not ice)
- Apr26 04/04, 18/04, 27/04 (3,200 / 4,000 / 4,000, all "NN ลูก" size-coded
  entries) -> COGS/Watermelon (owner confirmed these are watermelon buys)
- Apr26 24/04 barley/red-bean drink-mix (420) -> removed at owner's request
- May26 01/05 mixed umbrella/guava/milk/pump slip (7,823) split:
  700 COGS/Guava, 7,123 OPEX/Other
- May26 08/05 two water+coconut slips (4,555 + 2,820) -> COGS/Coconut Water
- May26 16/05 mixed police-fee/coconut/water/apple slip (4,290) split:
  2,000 OPEX/Other (police fee), 2,290 COGS/Coconut
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F321"/>
+  <dimension ref="A1:F323"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2243,10 +2243,10 @@
         <v>Feb26</v>
       </c>
       <c r="C56" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D56" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E56" t="str">
         <v>Unknown</v>
@@ -3686,7 +3686,7 @@
         <v>COGS</v>
       </c>
       <c r="D128" t="str">
-        <v>Ice</v>
+        <v>Watermelon</v>
       </c>
       <c r="E128" t="str">
         <v>4/4/68 40 ลูก</v>
@@ -4003,10 +4003,10 @@
         <v>Apr26</v>
       </c>
       <c r="C144" t="str">
-        <v>OPEX</v>
+        <v>COGS</v>
       </c>
       <c r="D144" t="str">
-        <v>Other</v>
+        <v>Watermelon</v>
       </c>
       <c r="E144" t="str">
         <v>16/4/2569</v>
@@ -4283,16 +4283,16 @@
         <v>Apr26</v>
       </c>
       <c r="C158" t="str">
-        <v>COGS</v>
+        <v>EXCLUDED</v>
       </c>
       <c r="D158" t="str">
-        <v>Other</v>
+        <v>Removed</v>
       </c>
       <c r="E158" t="str">
-        <v>บาร์เลย 4 ถั่วแดง 3 ถุงละ 60</v>
+        <v>บาร์เลย 4 ถั่วแดง 3 ถุงละ 60 (removed at owner request)</v>
       </c>
       <c r="F158">
-        <v>420</v>
+        <v>0</v>
       </c>
     </row>
     <row r="159">
@@ -4426,7 +4426,7 @@
         <v>COGS</v>
       </c>
       <c r="D165" t="str">
-        <v>Ice</v>
+        <v>Watermelon</v>
       </c>
       <c r="E165" t="str">
         <v>26/4/26 50 ลูก</v>
@@ -4749,10 +4749,10 @@
         <v>Guava</v>
       </c>
       <c r="E181" t="str">
-        <v>ร่ม 1176 ร่ม 843 ฝรั่ง 300 นมข้นจืด 785 ที่ปั้ม 176</v>
+        <v>ร่ม 1176 ร่ม 843 ฝรั่ง 300 นมข้นจืด 785 ที่ปั้ม 176 (Guava portion only)</v>
       </c>
       <c r="F181">
-        <v>7823</v>
+        <v>700</v>
       </c>
     </row>
     <row r="182">
@@ -5026,7 +5026,7 @@
         <v>COGS</v>
       </c>
       <c r="D195" t="str">
-        <v>Transportation</v>
+        <v>Coconut Water</v>
       </c>
       <c r="E195" t="str">
         <v>น้ำ 20 ขวด 900 ถอดเสื้อ 30 ลูก750 กล่องโฟม 3</v>
@@ -5066,7 +5066,7 @@
         <v>COGS</v>
       </c>
       <c r="D197" t="str">
-        <v>Water</v>
+        <v>Coconut Water</v>
       </c>
       <c r="E197" t="str">
         <v>6 พ.ค. น้ำ 30 ขวด 1500 บาท เนื้อ 11 โล 1320 บาท</v>
@@ -5523,16 +5523,16 @@
         <v>May26</v>
       </c>
       <c r="C220" t="str">
-        <v>COGS</v>
+        <v>OPEX</v>
       </c>
       <c r="D220" t="str">
-        <v>Ice</v>
+        <v>Other</v>
       </c>
       <c r="E220" t="str">
-        <v>Police fees -2000 2 head</v>
+        <v>Police fees (portion of mixed 16/05 slip)</v>
       </c>
       <c r="F220">
-        <v>4290</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="221">
@@ -7555,9 +7555,49 @@
         <v>486</v>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>01/05/2026</v>
+      </c>
+      <c r="B322" t="str">
+        <v>May26</v>
+      </c>
+      <c r="C322" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D322" t="str">
+        <v>Other</v>
+      </c>
+      <c r="E322" t="str">
+        <v>ร่ม+นมข้นจืด+ที่ปั้ม+ปืนฉีดน้ำ (remainder of mixed 01/05 slip, non-guava portion)</v>
+      </c>
+      <c r="F322">
+        <v>7123</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>16/05/2026</v>
+      </c>
+      <c r="B323" t="str">
+        <v>May26</v>
+      </c>
+      <c r="C323" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D323" t="str">
+        <v>Coconut</v>
+      </c>
+      <c r="E323" t="str">
+        <v>Coconut meat + water + apple (remainder of mixed 16/05 slip, non-police-fee portion)</v>
+      </c>
+      <c r="F323">
+        <v>2290</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F321"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F323"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: book March manager salary, close out remaining transfer questions
Owner confirmed B1's existing March Salary row (฿27,600 "ค่าแรงคนงาน Mar26")
is a different employee's wages, so the manager's ฿19,000 March salary
(matching the 05/03/2026 bank transfer) had never been booked. Added via
fix_march_salary.js, following the same dry-run/backup/idempotent pattern as
the other fix_*.js scripts; verified idempotent both standalone and via
test_idempotent.js.

Also folds in owner confirmation on the two remaining open transfers: the
02/02 ฿70,000 is B1's Feb rent + deposit (deposit correctly left unbooked,
same convention as B2's), and the ฿47,000 monthly transfers are rent + stock
as already documented. Only the ~฿280,000 manager-account receipts remain
open.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F464"/>
+  <dimension ref="A1:F465"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10415,9 +10415,29 @@
         <v>6000</v>
       </c>
     </row>
+    <row r="465">
+      <c r="A465" t="str">
+        <v>05/03/2026</v>
+      </c>
+      <c r="B465" t="str">
+        <v>Mar26</v>
+      </c>
+      <c r="C465" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D465" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E465" t="str">
+        <v>เงินเดือนเมน 3/26</v>
+      </c>
+      <c r="F465">
+        <v>19000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F464"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F465"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: book remaining manager-account slips, close out the audit
Owner supplied their own K PLR transaction notes for the 4 manager-account
slips: 20/02's 416 turned out already booked (split across two existing
rows that reconcile_bank.js's 1-to-1 matcher missed), and the other three
(27/02 equipment, 18/03 milk, 01/04 March salary for 3 employees) are now
booked via fix_manager_receipts_q1.js, following the established
dry-run/backup/idempotent pattern. Verified idempotent standalone and via
test_idempotent.js (now covering 7 fix scripts).

No open items remain in FINDINGS.md — every question raised during this
audit has been traced back to source and resolved with the owner.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -1168,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F465"/>
+  <dimension ref="A1:F468"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10435,9 +10435,69 @@
         <v>19000</v>
       </c>
     </row>
+    <row r="466">
+      <c r="A466" t="str">
+        <v>27/02/2026</v>
+      </c>
+      <c r="B466" t="str">
+        <v>Feb26</v>
+      </c>
+      <c r="C466" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D466" t="str">
+        <v>Investment</v>
+      </c>
+      <c r="E466" t="str">
+        <v>อุปกรณ์ (จากสลิปโอนผู้จัดการ)</v>
+      </c>
+      <c r="F466">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="B467" t="str">
+        <v>Mar26</v>
+      </c>
+      <c r="C467" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D467" t="str">
+        <v>Milk/Conden</v>
+      </c>
+      <c r="E467" t="str">
+        <v>นม + นมข้นหวาน (จากสลิปโอนผู้จัดการ)</v>
+      </c>
+      <c r="F467">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="str">
+        <v>01/04/2026</v>
+      </c>
+      <c r="B468" t="str">
+        <v>Apr26</v>
+      </c>
+      <c r="C468" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D468" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E468" t="str">
+        <v>เงินเดือนพนักงาน 3 คน มี.ค. 26</v>
+      </c>
+      <c r="F468">
+        <v>24600</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F465"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F468"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: recategorise the ฿7,700 Mar26 watermelon row filed under Orange
The row reads "แตงโม 51 ยอด3,500" but sat in COGS/Orange, so ฿7,700 of watermelon
cost was being allocated on orange usage. Owner confirmed the miscategorisation
and asked for it to be corrected despite Mar26 being one of his hand-kept months.

Mar26 orange spend drops 85,933 -> 78,233; watermelon picks it up. Orange's
per-kilo series is unaffected (the row carried no parseable quantity either way).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01492PXZhK4EeViAZZ2GAEhP
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -2926,10 +2926,10 @@
         <v>COGS</v>
       </c>
       <c r="D90" t="str">
-        <v>Orange</v>
+        <v>Watermelon</v>
       </c>
       <c r="E90" t="str">
-        <v>แตงโม 51 ยอด3,500</v>
+        <v>แตงโม 51 ยอด3,500 (แก้หมวด: เดิมลง Orange ผิด)</v>
       </c>
       <c r="F90">
         <v>7700</v>

</xml_diff>